<commit_message>
replacing ts_priceChange with p_gn('price')
</commit_message>
<xml_diff>
--- a/src_files/data_files/ObservedTrends.xlsx
+++ b/src_files/data_files/ObservedTrends.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BB\bb-master\north_european_model\src_files\data_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93F6FDD8-5400-4CFF-9E90-CD25D140FB28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30821A77-E233-4909-8A3D-C16EC2EE6A65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="770" firstSheet="6" activeTab="12" xr2:uid="{FFD27B4C-068C-4319-9C46-FFCA72C83648}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="770" firstSheet="6" activeTab="15" xr2:uid="{FFD27B4C-068C-4319-9C46-FFCA72C83648}"/>
   </bookViews>
   <sheets>
     <sheet name="VRE cap - ENTSOE NT2030" sheetId="7" r:id="rId1"/>
@@ -1748,6 +1748,89 @@
   </cellStyles>
   <dxfs count="18">
     <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor theme="0" tint="-0.14999847407452621"/>
@@ -1885,89 +1968,6 @@
         <top/>
         <bottom/>
       </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-        <scheme val="none"/>
-      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -3974,7 +3974,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{091DB227-DDC4-472D-997A-DFFFE388BE8E}" name="Table6" displayName="Table6" ref="A1:H185" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{091DB227-DDC4-472D-997A-DFFFE388BE8E}" name="Table6" displayName="Table6" ref="A1:H185" totalsRowShown="0" headerRowDxfId="17" headerRowBorderDxfId="16" tableBorderDxfId="15">
   <autoFilter ref="A1:H185" xr:uid="{B440C99F-3BB1-4A8C-9867-FC60A58307DE}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{4D600E68-4859-4617-99C0-EA7B63208C31}" name="grid"/>
@@ -3991,29 +3991,29 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E20E85B3-70B8-42FA-A4DB-D01011C9C779}" name="Table3" displayName="Table3" ref="A1:E154" totalsRowShown="0" headerRowDxfId="8" dataDxfId="6" headerRowBorderDxfId="7" tableBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E20E85B3-70B8-42FA-A4DB-D01011C9C779}" name="Table3" displayName="Table3" ref="A1:E154" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11">
   <autoFilter ref="A1:E154" xr:uid="{E20E85B3-70B8-42FA-A4DB-D01011C9C779}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{9E8A91B3-5637-47C2-B0AE-8BCDAB50C806}" name="Country" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{41E09046-0D25-4DEB-9887-2ECB6AE473F2}" name="Generator_ID" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{5500E0F2-38FA-425D-A49B-9DFF7856120F}" name="Scenario" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{2F7FD309-B9BB-4C5B-B61A-862D1DC7A785}" name="Year" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{278785FB-0A20-4E0A-8E84-551D5FDF9FC2}" name="capacity_output1" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{9E8A91B3-5637-47C2-B0AE-8BCDAB50C806}" name="Country" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{41E09046-0D25-4DEB-9887-2ECB6AE473F2}" name="Generator_ID" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{5500E0F2-38FA-425D-A49B-9DFF7856120F}" name="Scenario" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{2F7FD309-B9BB-4C5B-B61A-862D1DC7A785}" name="Year" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{278785FB-0A20-4E0A-8E84-551D5FDF9FC2}" name="capacity_output1" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6EBB9830-FC23-4A98-9C08-0AAF69FC2331}" name="Table8" displayName="Table8" ref="A1:F21" totalsRowShown="0" headerRowDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6EBB9830-FC23-4A98-9C08-0AAF69FC2331}" name="Table8" displayName="Table8" ref="A1:F21" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="A1:F21" xr:uid="{D9844F2F-2EE0-434B-9492-0280A28AB057}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{46AB9A07-935D-4BDF-BDAD-833C2B08B5EA}" name="Scenario" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{46AB9A07-935D-4BDF-BDAD-833C2B08B5EA}" name="Scenario" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{9C0117C3-729A-4483-9D40-255263DE774C}" name="Year"/>
-    <tableColumn id="3" xr3:uid="{F8AC0906-AF4C-4DB5-A628-E0D92C5871CF}" name="grid" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{5DE58EB2-B819-4C37-B8D5-9DAA3695DA87}" name="Country" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{2FBFC74F-134A-4E2A-8A69-7E943A399965}" name="price" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{78F6DB46-B023-4964-AA01-C06A0F1B985D}" name="emission_CO2" dataDxfId="12">
+    <tableColumn id="3" xr3:uid="{F8AC0906-AF4C-4DB5-A628-E0D92C5871CF}" name="grid" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{5DE58EB2-B819-4C37-B8D5-9DAA3695DA87}" name="Country" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{2FBFC74F-134A-4E2A-8A69-7E943A399965}" name="price" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{78F6DB46-B023-4964-AA01-C06A0F1B985D}" name="emission_CO2" dataDxfId="0">
       <calculatedColumnFormula>IFERROR(VLOOKUP($C2, [1]data_fuelEmissions!$D$4:$F$14,3,FALSE), 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>

</xml_diff>

<commit_message>
src_files: mark helper rows and columns with ##
The row marker was a single #, which is how every Excel error value starts, so
a broken formula silently deleted the row it sat in. Migrates the 18 comment
rows to ## and marks 54 helper columns, which the reader now drops by header
prefix rather than by the single hardcoded name "note".

Committed before the code change that reads ##: a cell reading "## PV" still
starts with #, so both the old rule and the new one skip it, and no commit in
between leaves the workbooks misread.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src_files/data_files/ObservedTrends.xlsx
+++ b/src_files/data_files/ObservedTrends.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BB\bb-master\north_european_model\src_files\data_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BB\bb-dev\north_european_model\src_files\data_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{978AE20D-20F3-42C2-A4B7-A21314830BB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C9DA93E-C666-4AA5-9F89-E5B85EE617C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="801" xr2:uid="{FFD27B4C-068C-4319-9C46-FFCA72C83648}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="801" firstSheet="3" activeTab="10" xr2:uid="{FFD27B4C-068C-4319-9C46-FFCA72C83648}"/>
   </bookViews>
   <sheets>
     <sheet name="vomcost mult" sheetId="20" r:id="rId1"/>
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2965" uniqueCount="327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3010" uniqueCount="328">
   <si>
     <t>Installed wind power capacity</t>
   </si>
@@ -950,15 +950,6 @@
     <t>EUR/MWh</t>
   </si>
   <si>
-    <t># Tier 1</t>
-  </si>
-  <si>
-    <t># Tier 2</t>
-  </si>
-  <si>
-    <t># Tier 3</t>
-  </si>
-  <si>
     <t>emission_bioCO2</t>
   </si>
   <si>
@@ -1061,21 +1052,6 @@
     <t>region multiplier</t>
   </si>
   <si>
-    <t># PV</t>
-  </si>
-  <si>
-    <t># Onshore</t>
-  </si>
-  <si>
-    <t># Offshore</t>
-  </si>
-  <si>
-    <t># Copying discharger capacity from charger capacity</t>
-  </si>
-  <si>
-    <t># Query charger capacity from previous sheets</t>
-  </si>
-  <si>
     <t>cost index 1</t>
   </si>
   <si>
@@ -1108,6 +1084,33 @@
   <si>
     <t>https://greenpowerdenmark.dk/nyheder/danmarks-stoerste-batteri-leverer-systemydelser-til-elnettet</t>
   </si>
+  <si>
+    <t>## Onshore</t>
+  </si>
+  <si>
+    <t>## Offshore</t>
+  </si>
+  <si>
+    <t>## PV</t>
+  </si>
+  <si>
+    <t>## Query charger capacity from previous sheets</t>
+  </si>
+  <si>
+    <t>##</t>
+  </si>
+  <si>
+    <t>## Copying discharger capacity from charger capacity</t>
+  </si>
+  <si>
+    <t>## Tier 1</t>
+  </si>
+  <si>
+    <t>## Tier 2</t>
+  </si>
+  <si>
+    <t>## Tier 3</t>
+  </si>
 </sst>
 </file>
 
@@ -1115,7 +1118,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.##########"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -1555,7 +1558,7 @@
     <xf numFmtId="9" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1730,7 +1733,7 @@
     <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
@@ -1758,6 +1761,11 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1787,8 +1795,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1799,16 +1805,6 @@
     <cellStyle name="Standard_Data provided by OT3" xfId="2" xr:uid="{CF5A235E-FF11-451C-B874-DD8F77BDC2C9}"/>
   </cellStyles>
   <dxfs count="40">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1894,61 +1890,31 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="left" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -1956,14 +1922,6 @@
           <color auto="1"/>
         </top>
       </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <border outline="0">
@@ -1986,15 +1944,8 @@
         <sz val="11"/>
         <color auto="1"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="none"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="7"/>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
@@ -2006,6 +1957,16 @@
         <top/>
         <bottom/>
       </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -2119,31 +2080,61 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="left" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <border outline="0">
@@ -2151,6 +2142,14 @@
           <color auto="1"/>
         </top>
       </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <border outline="0">
@@ -2173,8 +2172,15 @@
         <sz val="11"/>
         <color auto="1"/>
         <name val="Calibri"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="7"/>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
@@ -4797,6 +4803,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="fueldata"/>
@@ -4927,21 +4934,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E20E85B3-70B8-42FA-A4DB-D01011C9C779}" name="Table3" displayName="Table3" ref="A1:G104" totalsRowShown="0" headerRowDxfId="27" dataDxfId="25" headerRowBorderDxfId="26" tableBorderDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E20E85B3-70B8-42FA-A4DB-D01011C9C779}" name="Table3" displayName="Table3" ref="A1:G104" totalsRowShown="0" headerRowDxfId="28" dataDxfId="26" headerRowBorderDxfId="27" tableBorderDxfId="25">
   <autoFilter ref="A1:G104" xr:uid="{E20E85B3-70B8-42FA-A4DB-D01011C9C779}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F104">
     <sortCondition ref="A1:A104"/>
   </sortState>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{9E8A91B3-5637-47C2-B0AE-8BCDAB50C806}" name="Country" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{41E09046-0D25-4DEB-9887-2ECB6AE473F2}" name="Generator_ID" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{5500E0F2-38FA-425D-A49B-9DFF7856120F}" name="Scenario" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{2F7FD309-B9BB-4C5B-B61A-862D1DC7A785}" name="Year" dataDxfId="20"/>
-    <tableColumn id="5" xr3:uid="{278785FB-0A20-4E0A-8E84-551D5FDF9FC2}" name="capacity_output1" dataDxfId="19"/>
-    <tableColumn id="6" xr3:uid="{E48C78BB-51CD-490E-8B43-C4B84C6DDF67}" name="vomCosts" dataDxfId="18">
-      <calculatedColumnFormula>ROUND( VLOOKUP($B2,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A2,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{9E8A91B3-5637-47C2-B0AE-8BCDAB50C806}" name="Country" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{41E09046-0D25-4DEB-9887-2ECB6AE473F2}" name="Generator_ID" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{5500E0F2-38FA-425D-A49B-9DFF7856120F}" name="Scenario" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{2F7FD309-B9BB-4C5B-B61A-862D1DC7A785}" name="Year" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{278785FB-0A20-4E0A-8E84-551D5FDF9FC2}" name="capacity_output1" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{E48C78BB-51CD-490E-8B43-C4B84C6DDF67}" name="vomCosts" dataDxfId="19">
+      <calculatedColumnFormula>ROUND( VLOOKUP($B2,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A2,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{D44E8CC1-3697-402B-8C4C-49C226851A8A}" name="method" dataDxfId="0">
+    <tableColumn id="7" xr3:uid="{D44E8CC1-3697-402B-8C4C-49C226851A8A}" name="method" dataDxfId="18">
       <calculatedColumnFormula>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4950,18 +4957,18 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{3889FA67-DEB7-4516-91A9-7CF17095E2EC}" name="Table4" displayName="Table4" ref="A1:G70" totalsRowShown="0" headerRowDxfId="17" dataDxfId="15" headerRowBorderDxfId="16" tableBorderDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{3889FA67-DEB7-4516-91A9-7CF17095E2EC}" name="Table4" displayName="Table4" ref="A1:G70" totalsRowShown="0" headerRowDxfId="39" dataDxfId="37" headerRowBorderDxfId="38" tableBorderDxfId="36">
   <autoFilter ref="A1:G70" xr:uid="{3889FA67-DEB7-4516-91A9-7CF17095E2EC}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{E45B6B69-99E0-46CC-B622-954E9F00977C}" name="Country" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{0C46E4F6-5176-430E-8288-0E4AD27B50FB}" name="Generator_ID" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{23013750-786E-46E4-BB5A-5093E68C9E50}" name="Scenario" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{34290B83-B2CB-4767-BBB2-F1BACB31B343}" name="Year" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{C5354F01-9DC1-45FC-9DAC-9FEB4789196D}" name="capacity_output1" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{4BC02F33-D1CC-4D1B-829D-EC13C6E66759}" name="vomCosts" dataDxfId="8">
+    <tableColumn id="1" xr3:uid="{E45B6B69-99E0-46CC-B622-954E9F00977C}" name="Country" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{0C46E4F6-5176-430E-8288-0E4AD27B50FB}" name="Generator_ID" dataDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{23013750-786E-46E4-BB5A-5093E68C9E50}" name="Scenario" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{34290B83-B2CB-4767-BBB2-F1BACB31B343}" name="Year" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{C5354F01-9DC1-45FC-9DAC-9FEB4789196D}" name="capacity_output1" dataDxfId="31"/>
+    <tableColumn id="6" xr3:uid="{4BC02F33-D1CC-4D1B-829D-EC13C6E66759}" name="vomCosts" dataDxfId="30">
       <calculatedColumnFormula>400+V5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{44CC38D0-922B-47B3-AD5D-D98AD32D8306}" name="method" dataDxfId="7">
+    <tableColumn id="7" xr3:uid="{44CC38D0-922B-47B3-AD5D-D98AD32D8306}" name="method" dataDxfId="29">
       <calculatedColumnFormula>IF(Table4[[#This Row],[capacity_output1]]&lt;10, "remove", "")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4970,20 +4977,20 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{091DB227-DDC4-472D-997A-DFFFE388BE8E}" name="Table6" displayName="Table6" ref="A1:I93" totalsRowShown="0" headerRowDxfId="39" headerRowBorderDxfId="38" tableBorderDxfId="37">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{091DB227-DDC4-472D-997A-DFFFE388BE8E}" name="Table6" displayName="Table6" ref="A1:I93" totalsRowShown="0" headerRowDxfId="17" headerRowBorderDxfId="16" tableBorderDxfId="15">
   <autoFilter ref="A1:I93" xr:uid="{B440C99F-3BB1-4A8C-9867-FC60A58307DE}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{4D600E68-4859-4617-99C0-EA7B63208C31}" name="grid" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{55683E09-DD2F-48C0-AB3E-CC91087C7173}" name="from_country" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{C8327C88-FBE8-4FC2-A619-A4BA01413A1C}" name="to_country" dataDxfId="34"/>
-    <tableColumn id="4" xr3:uid="{742C6874-D199-4EE2-A562-EA0C285890D2}" name="scenario" dataDxfId="33"/>
-    <tableColumn id="5" xr3:uid="{1268EAAB-42FE-4A83-98BF-F41F14FEF437}" name="Year" dataDxfId="32"/>
-    <tableColumn id="6" xr3:uid="{DD03EC9C-1908-4818-A7AD-696B46FD7E55}" name="transferCap" dataDxfId="31"/>
-    <tableColumn id="8" xr3:uid="{858FE1C4-CAB1-497D-B42D-428703C91594}" name="variableTransCost" dataDxfId="30">
-      <calculatedColumnFormula>M2</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{4D600E68-4859-4617-99C0-EA7B63208C31}" name="grid" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{55683E09-DD2F-48C0-AB3E-CC91087C7173}" name="from_country" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{C8327C88-FBE8-4FC2-A619-A4BA01413A1C}" name="to_country" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{742C6874-D199-4EE2-A562-EA0C285890D2}" name="scenario" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{1268EAAB-42FE-4A83-98BF-F41F14FEF437}" name="Year" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{DD03EC9C-1908-4818-A7AD-696B46FD7E55}" name="transferCap" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{858FE1C4-CAB1-497D-B42D-428703C91594}" name="variableTransCost" dataDxfId="8">
+      <calculatedColumnFormula>M3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{BEFF1833-3A5D-4270-8A18-81866BBAA2B1}" name="transferLoss" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{B1909AD5-E5F0-4095-9C30-EDBB8410D520}" name="method" dataDxfId="28">
+    <tableColumn id="9" xr3:uid="{BEFF1833-3A5D-4270-8A18-81866BBAA2B1}" name="transferLoss" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{B1909AD5-E5F0-4095-9C30-EDBB8410D520}" name="method" dataDxfId="6">
       <calculatedColumnFormula>IF(Table6[[#This Row],[transferCap]]&lt;10, "remove", "")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4992,15 +4999,15 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6EBB9830-FC23-4A98-9C08-0AAF69FC2331}" name="Table8" displayName="Table8" ref="A1:F11" totalsRowShown="0" headerRowDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6EBB9830-FC23-4A98-9C08-0AAF69FC2331}" name="Table8" displayName="Table8" ref="A1:F11" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="A1:F11" xr:uid="{D9844F2F-2EE0-434B-9492-0280A28AB057}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{46AB9A07-935D-4BDF-BDAD-833C2B08B5EA}" name="Scenario" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{46AB9A07-935D-4BDF-BDAD-833C2B08B5EA}" name="Scenario" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{9C0117C3-729A-4483-9D40-255263DE774C}" name="Year"/>
-    <tableColumn id="3" xr3:uid="{F8AC0906-AF4C-4DB5-A628-E0D92C5871CF}" name="grid" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{5DE58EB2-B819-4C37-B8D5-9DAA3695DA87}" name="Country" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{2FBFC74F-134A-4E2A-8A69-7E943A399965}" name="price" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{78F6DB46-B023-4964-AA01-C06A0F1B985D}" name="emission_CO2" dataDxfId="1">
+    <tableColumn id="3" xr3:uid="{F8AC0906-AF4C-4DB5-A628-E0D92C5871CF}" name="grid" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{5DE58EB2-B819-4C37-B8D5-9DAA3695DA87}" name="Country" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{2FBFC74F-134A-4E2A-8A69-7E943A399965}" name="price" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{78F6DB46-B023-4964-AA01-C06A0F1B985D}" name="emission_CO2" dataDxfId="0">
       <calculatedColumnFormula>IFERROR(VLOOKUP($C2, [2]data_fuelEmissions!$D$4:$F$14,3,FALSE), 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5339,7 +5346,7 @@
   <sheetData>
     <row r="1" spans="1:18">
       <c r="A1" s="27" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="2" spans="1:18">
@@ -5347,7 +5354,7 @@
         <v>146</v>
       </c>
       <c r="B2" s="28" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -5355,7 +5362,7 @@
         <v>147</v>
       </c>
       <c r="B3" s="27" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5" spans="1:18">
@@ -5371,15 +5378,15 @@
         <v>150</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
     </row>
     <row r="7" spans="1:18">
       <c r="A7" s="28" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
     <row r="9" spans="1:18">
@@ -5399,7 +5406,7 @@
         <v>156</v>
       </c>
       <c r="F9" s="36" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="10" spans="1:18">
@@ -5422,16 +5429,16 @@
         <v>152</v>
       </c>
       <c r="J10" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="O10" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="P10" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="Q10" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="R10" s="23" t="s">
         <v>271</v>
@@ -5477,7 +5484,7 @@
     </row>
     <row r="12" spans="1:18">
       <c r="A12" s="32" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="B12" s="33">
         <v>33160</v>
@@ -5515,7 +5522,7 @@
     </row>
     <row r="13" spans="1:18">
       <c r="A13" s="32" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="B13" s="35">
         <v>33610</v>
@@ -5632,7 +5639,7 @@
     </row>
     <row r="16" spans="1:18">
       <c r="A16" s="32" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="B16" s="33">
         <v>20980</v>
@@ -6349,7 +6356,7 @@
         <v>72</v>
       </c>
       <c r="N34" s="17" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="O34" s="37">
         <f>F11</f>
@@ -6587,7 +6594,7 @@
     </row>
     <row r="46" spans="1:15">
       <c r="A46" s="32" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="B46" s="33">
         <v>33840</v>
@@ -6717,35 +6724,35 @@
     </row>
     <row r="55" spans="1:6">
       <c r="A55" s="28" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="28" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="57" spans="1:6">
       <c r="A57" s="28" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="28" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
     </row>
     <row r="62" spans="1:6">
       <c r="A62" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="B62" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
     </row>
     <row r="63" spans="1:6">
       <c r="A63" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B63" s="74">
         <v>46077</v>
@@ -6753,23 +6760,23 @@
     </row>
     <row r="65" spans="1:10">
       <c r="A65" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="B65" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="B66" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
     </row>
     <row r="69" spans="1:10">
       <c r="A69" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="B69" t="s">
         <v>153</v>
@@ -6784,7 +6791,7 @@
         <v>156</v>
       </c>
       <c r="F69" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="70" spans="1:10">
@@ -6829,7 +6836,7 @@
     </row>
     <row r="73" spans="1:10">
       <c r="A73" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="B73">
         <v>1.1422000000000001</v>
@@ -6847,12 +6854,12 @@
         <v>1.0824</v>
       </c>
       <c r="H73" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
     </row>
     <row r="75" spans="1:10">
       <c r="A75" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="B75">
         <f>ROUND(B70/B$73,0)</f>
@@ -6880,7 +6887,7 @@
     </row>
     <row r="76" spans="1:10">
       <c r="A76" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="B76">
         <f t="shared" ref="B76:F76" si="4">ROUND(B71/B$73,0)</f>
@@ -6948,10 +6955,37 @@
       <c r="G1" s="39" t="s">
         <v>167</v>
       </c>
+      <c r="K1" t="s">
+        <v>323</v>
+      </c>
+      <c r="L1" t="s">
+        <v>323</v>
+      </c>
+      <c r="M1" t="s">
+        <v>323</v>
+      </c>
+      <c r="N1" t="s">
+        <v>323</v>
+      </c>
+      <c r="O1" t="s">
+        <v>323</v>
+      </c>
+      <c r="P1" t="s">
+        <v>323</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>323</v>
+      </c>
+      <c r="R1" t="s">
+        <v>323</v>
+      </c>
+      <c r="S1" t="s">
+        <v>323</v>
+      </c>
     </row>
     <row r="2" spans="1:19">
       <c r="A2" s="17" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="B2" s="76"/>
       <c r="C2" s="76"/>
@@ -7333,7 +7367,7 @@
         <v>2000</v>
       </c>
       <c r="S13" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
     </row>
     <row r="14" spans="1:19">
@@ -7479,7 +7513,7 @@
         <v>350</v>
       </c>
       <c r="S16" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
     </row>
     <row r="17" spans="1:17">
@@ -8592,7 +8626,7 @@
     </row>
     <row r="47" spans="1:19">
       <c r="A47" s="17" t="s">
-        <v>314</v>
+        <v>324</v>
       </c>
       <c r="C47" s="19"/>
       <c r="D47" s="19"/>
@@ -10104,7 +10138,7 @@
   <sheetPr>
     <tabColor theme="6" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:M104"/>
+  <dimension ref="A1:N104"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.140625" customWidth="1"/>
@@ -10117,7 +10151,7 @@
     <col min="12" max="12" width="29.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" s="52" t="s">
         <v>3</v>
       </c>
@@ -10139,11 +10173,20 @@
       <c r="G1" s="52" t="s">
         <v>167</v>
       </c>
+      <c r="K1" t="s">
+        <v>323</v>
+      </c>
+      <c r="L1" t="s">
+        <v>323</v>
+      </c>
       <c r="M1" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
+        <v>323</v>
+      </c>
+      <c r="N1" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
         <v>111</v>
       </c>
@@ -10160,22 +10203,15 @@
         <v>113</v>
       </c>
       <c r="F2" s="19">
-        <f>ROUND( VLOOKUP($B2,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A2,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B2,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A2,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.93</v>
       </c>
       <c r="G2" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L2" s="60" t="s">
-        <v>190</v>
-      </c>
-      <c r="M2">
-        <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, $L2)</f>
-        <v>2.6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>111</v>
       </c>
@@ -10192,22 +10228,15 @@
         <v>356.5</v>
       </c>
       <c r="F3" s="19">
-        <f>ROUND( VLOOKUP($B3,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A3,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B3,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A3,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.93</v>
       </c>
       <c r="G3" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L3" t="s">
-        <v>191</v>
-      </c>
-      <c r="M3">
-        <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L3)</f>
-        <v>2.6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>111</v>
       </c>
@@ -10224,22 +10253,18 @@
         <v>220</v>
       </c>
       <c r="F4" s="19">
-        <f>ROUND( VLOOKUP($B4,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A4,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B4,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A4,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.93</v>
       </c>
       <c r="G4" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L4" s="60" t="s">
-        <v>192</v>
-      </c>
-      <c r="M4">
-        <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L4)</f>
-        <v>2.6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
+      <c r="M4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
         <v>111</v>
       </c>
@@ -10256,22 +10281,22 @@
         <v>370</v>
       </c>
       <c r="F5" s="19">
-        <f>ROUND( VLOOKUP($B5,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A5,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B5,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A5,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.93</v>
       </c>
       <c r="G5" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L5" t="s">
-        <v>194</v>
+      <c r="L5" s="60" t="s">
+        <v>190</v>
       </c>
       <c r="M5">
-        <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L5)</f>
+        <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, $L5)</f>
         <v>2.6</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
         <v>111</v>
       </c>
@@ -10288,22 +10313,22 @@
         <v>1751.6</v>
       </c>
       <c r="F6" s="19">
-        <f>ROUND( VLOOKUP($B6,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A6,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B6,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A6,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.93</v>
       </c>
       <c r="G6" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L6" s="60" t="s">
-        <v>195</v>
+      <c r="L6" t="s">
+        <v>191</v>
       </c>
       <c r="M6">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L6)</f>
         <v>2.6</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:14">
       <c r="A7" t="s">
         <v>111</v>
       </c>
@@ -10320,22 +10345,22 @@
         <v>51.2</v>
       </c>
       <c r="F7" s="19">
-        <f>ROUND( VLOOKUP($B7,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A7,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B7,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A7,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.93</v>
       </c>
       <c r="G7" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L7" t="s">
-        <v>198</v>
+      <c r="L7" s="60" t="s">
+        <v>192</v>
       </c>
       <c r="M7">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L7)</f>
         <v>2.6</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:14">
       <c r="A8" t="s">
         <v>111</v>
       </c>
@@ -10352,22 +10377,22 @@
         <v>17.2</v>
       </c>
       <c r="F8" s="19">
-        <f>ROUND( VLOOKUP($B8,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A8,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B8,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A8,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.93</v>
       </c>
       <c r="G8" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L8" s="60" t="s">
-        <v>199</v>
+      <c r="L8" t="s">
+        <v>194</v>
       </c>
       <c r="M8">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L8)</f>
         <v>2.6</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:14">
       <c r="A9" t="s">
         <v>111</v>
       </c>
@@ -10384,22 +10409,22 @@
         <v>414.3</v>
       </c>
       <c r="F9" s="19">
-        <f>ROUND( VLOOKUP($B9,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A9,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B9,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A9,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.37</v>
       </c>
       <c r="G9" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L9" t="s">
-        <v>196</v>
+      <c r="L9" s="60" t="s">
+        <v>195</v>
       </c>
       <c r="M9">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L9)</f>
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
       <c r="A10" t="s">
         <v>111</v>
       </c>
@@ -10416,22 +10441,22 @@
         <v>79.5</v>
       </c>
       <c r="F10" s="19">
-        <f>ROUND( VLOOKUP($B10,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A10,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B10,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A10,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.37</v>
       </c>
       <c r="G10" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L10" s="60" t="s">
-        <v>197</v>
+      <c r="L10" t="s">
+        <v>198</v>
       </c>
       <c r="M10">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L10)</f>
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
       <c r="A11" t="s">
         <v>111</v>
       </c>
@@ -10448,22 +10473,22 @@
         <v>120</v>
       </c>
       <c r="F11" s="19">
-        <f>ROUND( VLOOKUP($B11,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A11,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B11,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A11,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.37</v>
       </c>
       <c r="G11" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L11" t="s">
-        <v>207</v>
+      <c r="L11" s="60" t="s">
+        <v>199</v>
       </c>
       <c r="M11">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L11)</f>
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
       <c r="A12" t="s">
         <v>114</v>
       </c>
@@ -10480,22 +10505,22 @@
         <v>1775</v>
       </c>
       <c r="F12" s="19">
-        <f>ROUND( VLOOKUP($B12,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A12,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B12,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A12,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.91</v>
       </c>
       <c r="G12" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L12" s="60" t="s">
-        <v>201</v>
+      <c r="L12" t="s">
+        <v>196</v>
       </c>
       <c r="M12">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L12)</f>
-        <v>3.3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
       <c r="A13" t="s">
         <v>114</v>
       </c>
@@ -10512,22 +10537,22 @@
         <v>1732.1</v>
       </c>
       <c r="F13" s="19">
-        <f>ROUND( VLOOKUP($B13,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A13,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B13,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A13,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.91</v>
       </c>
       <c r="G13" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L13" t="s">
-        <v>204</v>
+      <c r="L13" s="60" t="s">
+        <v>197</v>
       </c>
       <c r="M13">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L13)</f>
-        <v>3.3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
       <c r="A14" t="s">
         <v>114</v>
       </c>
@@ -10544,21 +10569,22 @@
         <v>244</v>
       </c>
       <c r="F14" s="19">
-        <f>ROUND( VLOOKUP($B14,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A14,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B14,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A14,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.91</v>
       </c>
       <c r="G14" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L14" s="60" t="s">
-        <v>212</v>
+      <c r="L14" t="s">
+        <v>207</v>
       </c>
       <c r="M14">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13">
+        <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L14)</f>
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
       <c r="A15" t="s">
         <v>114</v>
       </c>
@@ -10575,22 +10601,22 @@
         <v>871</v>
       </c>
       <c r="F15" s="19">
-        <f>ROUND( VLOOKUP($B15,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A15,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B15,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A15,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.35</v>
       </c>
       <c r="G15" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L15" t="s">
-        <v>193</v>
+      <c r="L15" s="60" t="s">
+        <v>201</v>
       </c>
       <c r="M15">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L15)</f>
-        <v>2.6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
       <c r="A16" t="s">
         <v>114</v>
       </c>
@@ -10607,7 +10633,7 @@
         <v>354.4</v>
       </c>
       <c r="F16" s="19">
-        <f>ROUND( VLOOKUP($B16,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A16,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B16,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A16,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.7</v>
       </c>
       <c r="G16" s="19" t="str">
@@ -10615,7 +10641,7 @@
         <v/>
       </c>
       <c r="L16" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="M16">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L16)</f>
@@ -10639,7 +10665,7 @@
         <v>140</v>
       </c>
       <c r="F17" s="19">
-        <f>ROUND( VLOOKUP($B17,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A17,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B17,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A17,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.7</v>
       </c>
       <c r="G17" s="19" t="str">
@@ -10647,11 +10673,10 @@
         <v/>
       </c>
       <c r="L17" s="60" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="M17">
-        <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L17)</f>
-        <v>3.3</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -10671,19 +10696,19 @@
         <v>1765.5</v>
       </c>
       <c r="F18" s="19">
-        <f>ROUND( VLOOKUP($B18,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A18,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B18,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A18,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.36</v>
       </c>
       <c r="G18" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L18" s="60" t="s">
-        <v>200</v>
+      <c r="L18" t="s">
+        <v>193</v>
       </c>
       <c r="M18">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L18)</f>
-        <v>3.3</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="19" spans="1:13">
@@ -10703,15 +10728,15 @@
         <v>311.60000000000002</v>
       </c>
       <c r="F19" s="19">
-        <f>ROUND( VLOOKUP($B19,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A19,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B19,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A19,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.36</v>
       </c>
       <c r="G19" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L19" s="60" t="s">
-        <v>202</v>
+      <c r="L19" t="s">
+        <v>214</v>
       </c>
       <c r="M19">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L19)</f>
@@ -10735,15 +10760,15 @@
         <v>1011.5</v>
       </c>
       <c r="F20" s="19">
-        <f>ROUND( VLOOKUP($B20,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A20,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B20,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A20,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>4.37</v>
       </c>
       <c r="G20" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L20" t="s">
-        <v>203</v>
+      <c r="L20" s="60" t="s">
+        <v>215</v>
       </c>
       <c r="M20">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L20)</f>
@@ -10767,7 +10792,7 @@
         <v>178.5</v>
       </c>
       <c r="F21" s="19">
-        <f>ROUND( VLOOKUP($B21,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A21,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B21,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A21,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>4.37</v>
       </c>
       <c r="G21" s="19" t="str">
@@ -10775,7 +10800,7 @@
         <v/>
       </c>
       <c r="L21" s="60" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="M21">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L21)</f>
@@ -10799,15 +10824,15 @@
         <v>1620.4</v>
       </c>
       <c r="F22" s="19">
-        <f>ROUND( VLOOKUP($B22,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A22,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B22,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A22,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.88</v>
       </c>
       <c r="G22" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L22" t="s">
-        <v>211</v>
+      <c r="L22" s="60" t="s">
+        <v>202</v>
       </c>
       <c r="M22">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L22)</f>
@@ -10831,7 +10856,7 @@
         <v>53.6</v>
       </c>
       <c r="F23" s="19">
-        <f>ROUND( VLOOKUP($B23,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A23,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B23,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A23,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.88</v>
       </c>
       <c r="G23" s="19" t="str">
@@ -10839,11 +10864,11 @@
         <v/>
       </c>
       <c r="L23" t="s">
-        <v>187</v>
+        <v>203</v>
       </c>
       <c r="M23">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L23)</f>
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -10863,7 +10888,7 @@
         <v>460.4</v>
       </c>
       <c r="F24" s="19">
-        <f>ROUND( VLOOKUP($B24,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A24,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B24,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A24,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.88</v>
       </c>
       <c r="G24" s="19" t="str">
@@ -10871,7 +10896,7 @@
         <v/>
       </c>
       <c r="L24" s="60" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="M24">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L24)</f>
@@ -10895,15 +10920,15 @@
         <v>1658.6</v>
       </c>
       <c r="F25" s="19">
-        <f>ROUND( VLOOKUP($B25,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A25,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B25,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A25,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.88</v>
       </c>
       <c r="G25" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L25" s="60" t="s">
-        <v>210</v>
+      <c r="L25" t="s">
+        <v>211</v>
       </c>
       <c r="M25">
         <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L25)</f>
@@ -10927,18 +10952,19 @@
         <v>18452.900000000001</v>
       </c>
       <c r="F26" s="19">
-        <f>ROUND( VLOOKUP($B26,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A26,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B26,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A26,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.88</v>
       </c>
       <c r="G26" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="L26" s="60" t="s">
-        <v>229</v>
+      <c r="L26" t="s">
+        <v>187</v>
       </c>
       <c r="M26">
-        <v>3</v>
+        <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L26)</f>
+        <v>3.2</v>
       </c>
     </row>
     <row r="27" spans="1:13">
@@ -10958,13 +10984,20 @@
         <v>2355.8000000000002</v>
       </c>
       <c r="F27" s="19">
-        <f>ROUND( VLOOKUP($B27,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A27,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B27,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A27,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.88</v>
       </c>
       <c r="G27" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
+      <c r="L27" s="60" t="s">
+        <v>206</v>
+      </c>
+      <c r="M27">
+        <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L27)</f>
+        <v>3.3</v>
+      </c>
     </row>
     <row r="28" spans="1:13">
       <c r="A28" t="s">
@@ -10983,13 +11016,20 @@
         <v>43.3</v>
       </c>
       <c r="F28" s="19">
-        <f>ROUND( VLOOKUP($B28,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A28,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B28,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A28,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.88</v>
       </c>
       <c r="G28" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
+      <c r="L28" s="60" t="s">
+        <v>210</v>
+      </c>
+      <c r="M28">
+        <f>SUMIFS([1]unittypedata!$S:$S,[1]unittypedata!$C:$C, L28)</f>
+        <v>3.3</v>
+      </c>
     </row>
     <row r="29" spans="1:13">
       <c r="A29" t="s">
@@ -11008,13 +11048,19 @@
         <v>109.7</v>
       </c>
       <c r="F29" s="19">
-        <f>ROUND( VLOOKUP($B29,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A29,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B29,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A29,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.33</v>
       </c>
       <c r="G29" s="19" t="str">
         <f>IF(Table3[[#This Row],[capacity_output1]]&lt;10, "remove", "")</f>
         <v/>
       </c>
+      <c r="L29" s="60" t="s">
+        <v>229</v>
+      </c>
+      <c r="M29">
+        <v>3</v>
+      </c>
     </row>
     <row r="30" spans="1:13">
       <c r="A30" t="s">
@@ -11033,7 +11079,7 @@
         <v>945.1</v>
       </c>
       <c r="F30" s="19">
-        <f>ROUND( VLOOKUP($B30,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A30,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B30,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A30,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.33</v>
       </c>
       <c r="G30" s="19" t="str">
@@ -11058,7 +11104,7 @@
         <v>1585.3</v>
       </c>
       <c r="F31" s="19">
-        <f>ROUND( VLOOKUP($B31,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A31,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B31,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A31,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.33</v>
       </c>
       <c r="G31" s="19" t="str">
@@ -11083,7 +11129,7 @@
         <v>57.8</v>
       </c>
       <c r="F32" s="19">
-        <f>ROUND( VLOOKUP($B32,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A32,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B32,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A32,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.25</v>
       </c>
       <c r="G32" s="19" t="str">
@@ -11108,7 +11154,7 @@
         <v>54.6</v>
       </c>
       <c r="F33" s="19">
-        <f>ROUND( VLOOKUP($B33,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A33,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B33,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A33,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.25</v>
       </c>
       <c r="G33" s="19" t="str">
@@ -11133,7 +11179,7 @@
         <v>72</v>
       </c>
       <c r="F34" s="19">
-        <f>ROUND( VLOOKUP($B34,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A34,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B34,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A34,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.25</v>
       </c>
       <c r="G34" s="19" t="str">
@@ -11158,7 +11204,7 @@
         <v>103.1</v>
       </c>
       <c r="F35" s="19">
-        <f>ROUND( VLOOKUP($B35,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A35,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B35,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A35,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.25</v>
       </c>
       <c r="G35" s="19" t="str">
@@ -11183,7 +11229,7 @@
         <v>1165.5</v>
       </c>
       <c r="F36" s="19">
-        <f>ROUND( VLOOKUP($B36,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A36,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B36,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A36,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>4.13</v>
       </c>
       <c r="G36" s="19" t="str">
@@ -11208,7 +11254,7 @@
         <v>65.099999999999994</v>
       </c>
       <c r="F37" s="19">
-        <f>ROUND( VLOOKUP($B37,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A37,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B37,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A37,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>4.13</v>
       </c>
       <c r="G37" s="19" t="str">
@@ -11233,7 +11279,7 @@
         <v>531</v>
       </c>
       <c r="F38" s="19">
-        <f>ROUND( VLOOKUP($B38,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A38,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B38,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A38,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.63</v>
       </c>
       <c r="G38" s="19" t="str">
@@ -11258,7 +11304,7 @@
         <v>47.2</v>
       </c>
       <c r="F39" s="19">
-        <f>ROUND( VLOOKUP($B39,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A39,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B39,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A39,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.22</v>
       </c>
       <c r="G39" s="19" t="str">
@@ -11283,7 +11329,7 @@
         <v>54.3</v>
       </c>
       <c r="F40" s="19">
-        <f>ROUND( VLOOKUP($B40,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A40,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B40,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A40,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.22</v>
       </c>
       <c r="G40" s="19" t="str">
@@ -11308,7 +11354,7 @@
         <v>129.6</v>
       </c>
       <c r="F41" s="19">
-        <f>ROUND( VLOOKUP($B41,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A41,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B41,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A41,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.22</v>
       </c>
       <c r="G41" s="19" t="str">
@@ -11333,7 +11379,7 @@
         <v>69.7</v>
       </c>
       <c r="F42" s="19">
-        <f>ROUND( VLOOKUP($B42,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A42,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B42,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A42,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.22</v>
       </c>
       <c r="G42" s="19" t="str">
@@ -11358,7 +11404,7 @@
         <v>448.2</v>
       </c>
       <c r="F43" s="19">
-        <f>ROUND( VLOOKUP($B43,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A43,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B43,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A43,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.22</v>
       </c>
       <c r="G43" s="19" t="str">
@@ -11383,7 +11429,7 @@
         <v>111.7</v>
       </c>
       <c r="F44" s="19">
-        <f>ROUND( VLOOKUP($B44,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A44,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B44,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A44,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.6</v>
       </c>
       <c r="G44" s="19" t="str">
@@ -11408,7 +11454,7 @@
         <v>375.4</v>
       </c>
       <c r="F45" s="19">
-        <f>ROUND( VLOOKUP($B45,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A45,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B45,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A45,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.6</v>
       </c>
       <c r="G45" s="19" t="str">
@@ -11433,7 +11479,7 @@
         <v>778.1</v>
       </c>
       <c r="F46" s="19">
-        <f>ROUND( VLOOKUP($B46,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A46,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B46,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A46,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>4.09</v>
       </c>
       <c r="G46" s="19" t="str">
@@ -11458,7 +11504,7 @@
         <v>165.8</v>
       </c>
       <c r="F47" s="19">
-        <f>ROUND( VLOOKUP($B47,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A47,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B47,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A47,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.6</v>
       </c>
       <c r="G47" s="19" t="str">
@@ -11483,7 +11529,7 @@
         <v>250</v>
       </c>
       <c r="F48" s="19">
-        <f>ROUND( VLOOKUP($B48,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A48,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B48,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A48,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.0699999999999998</v>
       </c>
       <c r="G48" s="19" t="str">
@@ -11508,7 +11554,7 @@
         <v>658</v>
       </c>
       <c r="F49" s="19">
-        <f>ROUND( VLOOKUP($B49,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A49,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B49,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A49,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.63</v>
       </c>
       <c r="G49" s="19" t="str">
@@ -11533,7 +11579,7 @@
         <v>173</v>
       </c>
       <c r="F50" s="19">
-        <f>ROUND( VLOOKUP($B50,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A50,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B50,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A50,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.63</v>
       </c>
       <c r="G50" s="19" t="str">
@@ -11558,7 +11604,7 @@
         <v>24498</v>
       </c>
       <c r="F51" s="19">
-        <f>ROUND( VLOOKUP($B51,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A51,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B51,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A51,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.38</v>
       </c>
       <c r="G51" s="19" t="str">
@@ -11583,7 +11629,7 @@
         <v>4335.3</v>
       </c>
       <c r="F52" s="19">
-        <f>ROUND( VLOOKUP($B52,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A52,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B52,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A52,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.75</v>
       </c>
       <c r="G52" s="19" t="str">
@@ -11608,7 +11654,7 @@
         <v>765.1</v>
       </c>
       <c r="F53" s="19">
-        <f>ROUND( VLOOKUP($B53,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A53,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B53,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A53,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.75</v>
       </c>
       <c r="G53" s="19" t="str">
@@ -11633,7 +11679,7 @@
         <v>45</v>
       </c>
       <c r="F54" s="19">
-        <f>ROUND( VLOOKUP($B54,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A54,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B54,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A54,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.88</v>
       </c>
       <c r="G54" s="19" t="str">
@@ -11658,7 +11704,7 @@
         <v>640</v>
       </c>
       <c r="F55" s="19">
-        <f>ROUND( VLOOKUP($B55,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A55,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B55,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A55,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.88</v>
       </c>
       <c r="G55" s="19" t="str">
@@ -11683,7 +11729,7 @@
         <v>234</v>
       </c>
       <c r="F56" s="19">
-        <f>ROUND( VLOOKUP($B56,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A56,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B56,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A56,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.88</v>
       </c>
       <c r="G56" s="19" t="str">
@@ -11708,7 +11754,7 @@
         <v>87</v>
       </c>
       <c r="F57" s="19">
-        <f>ROUND( VLOOKUP($B57,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A57,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B57,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A57,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.88</v>
       </c>
       <c r="G57" s="19" t="str">
@@ -11733,7 +11779,7 @@
         <v>38</v>
       </c>
       <c r="F58" s="19">
-        <f>ROUND( VLOOKUP($B58,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A58,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B58,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A58,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.88</v>
       </c>
       <c r="G58" s="19" t="str">
@@ -11758,7 +11804,7 @@
         <v>1196</v>
       </c>
       <c r="F59" s="19">
-        <f>ROUND( VLOOKUP($B59,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A59,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B59,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A59,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.66</v>
       </c>
       <c r="G59" s="19" t="str">
@@ -11783,7 +11829,7 @@
         <v>3734.9</v>
       </c>
       <c r="F60" s="19">
-        <f>ROUND( VLOOKUP($B60,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A60,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B60,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A60,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.32</v>
       </c>
       <c r="G60" s="19" t="str">
@@ -11808,7 +11854,7 @@
         <v>659.1</v>
       </c>
       <c r="F61" s="19">
-        <f>ROUND( VLOOKUP($B61,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A61,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B61,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A61,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.32</v>
       </c>
       <c r="G61" s="19" t="str">
@@ -11833,7 +11879,7 @@
         <v>414</v>
       </c>
       <c r="F62" s="19">
-        <f>ROUND( VLOOKUP($B62,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A62,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B62,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A62,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.74</v>
       </c>
       <c r="G62" s="19" t="str">
@@ -11858,7 +11904,7 @@
         <v>792</v>
       </c>
       <c r="F63" s="19">
-        <f>ROUND( VLOOKUP($B63,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A63,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B63,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A63,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.74</v>
       </c>
       <c r="G63" s="19" t="str">
@@ -11883,7 +11929,7 @@
         <v>5347</v>
       </c>
       <c r="F64" s="19">
-        <f>ROUND( VLOOKUP($B64,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A64,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B64,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A64,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.74</v>
       </c>
       <c r="G64" s="19" t="str">
@@ -11908,7 +11954,7 @@
         <v>437</v>
       </c>
       <c r="F65" s="19">
-        <f>ROUND( VLOOKUP($B65,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A65,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B65,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A65,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.74</v>
       </c>
       <c r="G65" s="19" t="str">
@@ -11933,7 +11979,7 @@
         <v>199</v>
       </c>
       <c r="F66" s="19">
-        <f>ROUND( VLOOKUP($B66,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A66,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B66,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A66,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.74</v>
       </c>
       <c r="G66" s="19" t="str">
@@ -11958,7 +12004,7 @@
         <v>1255</v>
       </c>
       <c r="F67" s="19">
-        <f>ROUND( VLOOKUP($B67,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A67,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B67,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A67,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.21</v>
       </c>
       <c r="G67" s="19" t="str">
@@ -11983,7 +12029,7 @@
         <v>24704.400000000001</v>
       </c>
       <c r="F68" s="19">
-        <f>ROUND( VLOOKUP($B68,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A68,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B68,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A68,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.16</v>
       </c>
       <c r="G68" s="19" t="str">
@@ -12008,7 +12054,7 @@
         <v>37056.6</v>
       </c>
       <c r="F69" s="19">
-        <f>ROUND( VLOOKUP($B69,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A69,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B69,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A69,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.16</v>
       </c>
       <c r="G69" s="19" t="str">
@@ -12033,7 +12079,7 @@
         <v>510</v>
       </c>
       <c r="F70" s="19">
-        <f>ROUND( VLOOKUP($B70,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A70,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B70,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A70,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>1.99</v>
       </c>
       <c r="G70" s="19" t="str">
@@ -12058,7 +12104,7 @@
         <v>403</v>
       </c>
       <c r="F71" s="19">
-        <f>ROUND( VLOOKUP($B71,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A71,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B71,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A71,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>1.99</v>
       </c>
       <c r="G71" s="19" t="str">
@@ -12083,7 +12129,7 @@
         <v>110</v>
       </c>
       <c r="F72" s="19">
-        <f>ROUND( VLOOKUP($B72,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A72,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B72,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A72,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>1.61</v>
       </c>
       <c r="G72" s="19" t="str">
@@ -12108,7 +12154,7 @@
         <v>1004</v>
       </c>
       <c r="F73" s="19">
-        <f>ROUND( VLOOKUP($B73,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A73,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B73,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A73,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>1.82</v>
       </c>
       <c r="G73" s="19" t="str">
@@ -12133,7 +12179,7 @@
         <v>73</v>
       </c>
       <c r="F74" s="19">
-        <f>ROUND( VLOOKUP($B74,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A74,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B74,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A74,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>1.82</v>
       </c>
       <c r="G74" s="19" t="str">
@@ -12158,7 +12204,7 @@
         <v>2536.5</v>
       </c>
       <c r="F75" s="19">
-        <f>ROUND( VLOOKUP($B75,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A75,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B75,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A75,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.07</v>
       </c>
       <c r="G75" s="19" t="str">
@@ -12183,7 +12229,7 @@
         <v>7083</v>
       </c>
       <c r="F76" s="19">
-        <f>ROUND( VLOOKUP($B76,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A76,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B76,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A76,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.07</v>
       </c>
       <c r="G76" s="19" t="str">
@@ -12208,7 +12254,7 @@
         <v>314</v>
       </c>
       <c r="F77" s="19">
-        <f>ROUND( VLOOKUP($B77,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A77,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B77,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A77,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.07</v>
       </c>
       <c r="G77" s="19" t="str">
@@ -12233,7 +12279,7 @@
         <v>165</v>
       </c>
       <c r="F78" s="19">
-        <f>ROUND( VLOOKUP($B78,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A78,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B78,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A78,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.07</v>
       </c>
       <c r="G78" s="19" t="str">
@@ -12258,7 +12304,7 @@
         <v>413.1</v>
       </c>
       <c r="F79" s="19">
-        <f>ROUND( VLOOKUP($B79,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A79,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B79,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A79,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.54</v>
       </c>
       <c r="G79" s="19" t="str">
@@ -12283,7 +12329,7 @@
         <v>72.900000000000006</v>
       </c>
       <c r="F80" s="19">
-        <f>ROUND( VLOOKUP($B80,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A80,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B80,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A80,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.54</v>
       </c>
       <c r="G80" s="19" t="str">
@@ -12308,7 +12354,7 @@
         <v>9620.7000000000007</v>
       </c>
       <c r="F81" s="19">
-        <f>ROUND( VLOOKUP($B81,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A81,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B81,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A81,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>1.79</v>
       </c>
       <c r="G81" s="19" t="str">
@@ -12333,7 +12379,7 @@
         <v>1663</v>
       </c>
       <c r="F82" s="19">
-        <f>ROUND( VLOOKUP($B82,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A82,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B82,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A82,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.2799999999999998</v>
       </c>
       <c r="G82" s="19" t="str">
@@ -12358,7 +12404,7 @@
         <v>3305.5</v>
       </c>
       <c r="F83" s="19">
-        <f>ROUND( VLOOKUP($B83,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A83,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B83,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A83,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.2799999999999998</v>
       </c>
       <c r="G83" s="19" t="str">
@@ -12383,7 +12429,7 @@
         <v>5466.6</v>
       </c>
       <c r="F84" s="19">
-        <f>ROUND( VLOOKUP($B84,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A84,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B84,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A84,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.2799999999999998</v>
       </c>
       <c r="G84" s="19" t="str">
@@ -12408,7 +12454,7 @@
         <v>1872.1</v>
       </c>
       <c r="F85" s="19">
-        <f>ROUND( VLOOKUP($B85,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A85,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B85,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A85,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.2799999999999998</v>
       </c>
       <c r="G85" s="19" t="str">
@@ -12433,7 +12479,7 @@
         <v>4696</v>
       </c>
       <c r="F86" s="19">
-        <f>ROUND( VLOOKUP($B86,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A86,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B86,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A86,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.2799999999999998</v>
       </c>
       <c r="G86" s="19" t="str">
@@ -12458,7 +12504,7 @@
         <v>1824</v>
       </c>
       <c r="F87" s="19">
-        <f>ROUND( VLOOKUP($B87,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A87,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B87,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A87,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.2799999999999998</v>
       </c>
       <c r="G87" s="19" t="str">
@@ -12483,7 +12529,7 @@
         <v>97</v>
       </c>
       <c r="F88" s="19">
-        <f>ROUND( VLOOKUP($B88,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A88,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B88,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A88,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.07</v>
       </c>
       <c r="G88" s="19" t="str">
@@ -12508,7 +12554,7 @@
         <v>54</v>
       </c>
       <c r="F89" s="19">
-        <f>ROUND( VLOOKUP($B89,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A89,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B89,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A89,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.03</v>
       </c>
       <c r="G89" s="19" t="str">
@@ -12533,7 +12579,7 @@
         <v>5850.6</v>
       </c>
       <c r="F90" s="19">
-        <f>ROUND( VLOOKUP($B90,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A90,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B90,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A90,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.5</v>
       </c>
       <c r="G90" s="19" t="str">
@@ -12558,7 +12604,7 @@
         <v>1032.5</v>
       </c>
       <c r="F91" s="19">
-        <f>ROUND( VLOOKUP($B91,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A91,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B91,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A91,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.5</v>
       </c>
       <c r="G91" s="19" t="str">
@@ -12583,7 +12629,7 @@
         <v>4300</v>
       </c>
       <c r="F92" s="19">
-        <f>ROUND( VLOOKUP($B92,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A92,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B92,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A92,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.03</v>
       </c>
       <c r="G92" s="19" t="str">
@@ -12608,7 +12654,7 @@
         <v>539</v>
       </c>
       <c r="F93" s="19">
-        <f>ROUND( VLOOKUP($B93,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A93,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B93,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A93,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.03</v>
       </c>
       <c r="G93" s="19" t="str">
@@ -12633,7 +12679,7 @@
         <v>21988.5</v>
       </c>
       <c r="F94" s="19">
-        <f>ROUND( VLOOKUP($B94,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A94,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B94,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A94,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.03</v>
       </c>
       <c r="G94" s="19" t="str">
@@ -12658,7 +12704,7 @@
         <v>408</v>
       </c>
       <c r="F95" s="19">
-        <f>ROUND( VLOOKUP($B95,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A95,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B95,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A95,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.03</v>
       </c>
       <c r="G95" s="19" t="str">
@@ -12683,7 +12729,7 @@
         <v>2456.9</v>
       </c>
       <c r="F96" s="19">
-        <f>ROUND( VLOOKUP($B96,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A96,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B96,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A96,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.03</v>
       </c>
       <c r="G96" s="19" t="str">
@@ -12708,7 +12754,7 @@
         <v>2448.6999999999998</v>
       </c>
       <c r="F97" s="19">
-        <f>ROUND( VLOOKUP($B97,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A97,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B97,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A97,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.4500000000000002</v>
       </c>
       <c r="G97" s="19" t="str">
@@ -12733,7 +12779,7 @@
         <v>5062.1000000000004</v>
       </c>
       <c r="F98" s="19">
-        <f>ROUND( VLOOKUP($B98,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A98,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B98,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A98,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.4500000000000002</v>
       </c>
       <c r="G98" s="19" t="str">
@@ -12758,7 +12804,7 @@
         <v>204.7</v>
       </c>
       <c r="F99" s="19">
-        <f>ROUND( VLOOKUP($B99,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A99,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B99,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A99,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.84</v>
       </c>
       <c r="G99" s="19" t="str">
@@ -12783,7 +12829,7 @@
         <v>70.8</v>
       </c>
       <c r="F100" s="19">
-        <f>ROUND( VLOOKUP($B100,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A100,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B100,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A100,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.84</v>
       </c>
       <c r="G100" s="19" t="str">
@@ -12808,7 +12854,7 @@
         <v>389</v>
       </c>
       <c r="F101" s="19">
-        <f>ROUND( VLOOKUP($B101,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A101,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B101,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A101,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>2.4500000000000002</v>
       </c>
       <c r="G101" s="19" t="str">
@@ -12833,7 +12879,7 @@
         <v>18</v>
       </c>
       <c r="F102" s="19">
-        <f>ROUND( VLOOKUP($B102,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A102,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B102,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A102,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.84</v>
       </c>
       <c r="G102" s="19" t="str">
@@ -12858,7 +12904,7 @@
         <v>4683.5</v>
       </c>
       <c r="F103" s="19">
-        <f>ROUND( VLOOKUP($B103,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A103,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B103,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A103,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.5</v>
       </c>
       <c r="G103" s="19" t="str">
@@ -12883,7 +12929,7 @@
         <v>826.5</v>
       </c>
       <c r="F104" s="19">
-        <f>ROUND( VLOOKUP($B104,$L$2:$M$26, 2, FALSE) * (1+ VLOOKUP($A104,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
+        <f>ROUND( VLOOKUP($B104,$L$5:$M$29, 2, FALSE) * (1+ VLOOKUP($A104,'vomcost mult'!$N$10:$R$32,5, FALSE)), 2)</f>
         <v>3.5</v>
       </c>
       <c r="G104" s="19" t="str">
@@ -12945,10 +12991,85 @@
       <c r="G1" s="71" t="s">
         <v>167</v>
       </c>
+      <c r="I1" t="s">
+        <v>323</v>
+      </c>
+      <c r="J1" t="s">
+        <v>323</v>
+      </c>
+      <c r="K1" t="s">
+        <v>323</v>
+      </c>
+      <c r="L1" t="s">
+        <v>323</v>
+      </c>
+      <c r="M1" t="s">
+        <v>323</v>
+      </c>
+      <c r="N1" t="s">
+        <v>323</v>
+      </c>
+      <c r="O1" t="s">
+        <v>323</v>
+      </c>
+      <c r="P1" t="s">
+        <v>323</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>323</v>
+      </c>
+      <c r="R1" t="s">
+        <v>323</v>
+      </c>
+      <c r="S1" t="s">
+        <v>323</v>
+      </c>
+      <c r="T1" t="s">
+        <v>323</v>
+      </c>
+      <c r="U1" t="s">
+        <v>323</v>
+      </c>
+      <c r="V1" t="s">
+        <v>323</v>
+      </c>
+      <c r="W1" t="s">
+        <v>323</v>
+      </c>
+      <c r="X1" t="s">
+        <v>323</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>323</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>323</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>323</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>323</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>323</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>323</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>323</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>323</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>323</v>
+      </c>
     </row>
     <row r="2" spans="1:33">
       <c r="A2" s="17" t="s">
-        <v>274</v>
+        <v>325</v>
       </c>
       <c r="C2" s="19"/>
       <c r="D2" s="19"/>
@@ -14829,7 +14950,7 @@
     </row>
     <row r="25" spans="1:33">
       <c r="A25" s="17" t="s">
-        <v>275</v>
+        <v>326</v>
       </c>
       <c r="C25" s="19"/>
       <c r="D25" s="19"/>
@@ -15672,7 +15793,7 @@
     </row>
     <row r="48" spans="1:7">
       <c r="A48" s="17" t="s">
-        <v>276</v>
+        <v>327</v>
       </c>
       <c r="C48" s="19"/>
       <c r="D48" s="19"/>
@@ -16265,7 +16386,7 @@
   <sheetPr>
     <tabColor theme="6" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:Q93"/>
+  <dimension ref="A1:Q94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9" style="73" bestFit="1" customWidth="1"/>
@@ -16307,13 +16428,19 @@
         <v>167</v>
       </c>
       <c r="M1" t="s">
-        <v>278</v>
+        <v>323</v>
+      </c>
+      <c r="N1" t="s">
+        <v>323</v>
+      </c>
+      <c r="O1" t="s">
+        <v>323</v>
       </c>
       <c r="P1" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="Q1" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
     </row>
     <row r="2" spans="1:17">
@@ -16336,24 +16463,21 @@
         <v>1200</v>
       </c>
       <c r="G2" s="19">
-        <f>M2</f>
+        <f>M3</f>
         <v>2.6399999999999997</v>
       </c>
       <c r="I2" s="19" t="str">
         <f>IF(Table6[[#This Row],[transferCap]]&lt;10, "remove", "")</f>
         <v/>
       </c>
-      <c r="M2">
-        <f>ROUND(P2*Q2, 2)+1</f>
-        <v>2.6399999999999997</v>
-      </c>
-      <c r="P2">
-        <f>(1+ VLOOKUP($B2,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1280000000000001</v>
-      </c>
-      <c r="Q2">
-        <f>(1+ VLOOKUP($C2,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.456</v>
+      <c r="M2" t="s">
+        <v>275</v>
+      </c>
+      <c r="P2" t="s">
+        <v>308</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -16376,7 +16500,7 @@
         <v>1200</v>
       </c>
       <c r="G3" s="19">
-        <f t="shared" ref="G3:G66" si="0">M3</f>
+        <f t="shared" ref="G3:G66" si="0">M4</f>
         <v>2.6399999999999997</v>
       </c>
       <c r="I3" s="19" t="str">
@@ -16384,16 +16508,16 @@
         <v/>
       </c>
       <c r="M3">
-        <f t="shared" ref="M3:M66" si="1">ROUND(P3*Q3, 2)+1</f>
+        <f>ROUND(P3*Q3, 2)+1</f>
         <v>2.6399999999999997</v>
       </c>
       <c r="P3">
-        <f>(1+ VLOOKUP($B3,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B2,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1280000000000001</v>
+      </c>
+      <c r="Q3">
+        <f>(1+ VLOOKUP($C2,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.456</v>
-      </c>
-      <c r="Q3">
-        <f>(1+ VLOOKUP($C3,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1280000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -16424,16 +16548,16 @@
         <v/>
       </c>
       <c r="M4">
-        <f t="shared" si="1"/>
-        <v>2.25</v>
+        <f t="shared" ref="M4:M67" si="1">ROUND(P4*Q4, 2)+1</f>
+        <v>2.6399999999999997</v>
       </c>
       <c r="P4">
-        <f>(1+ VLOOKUP($B4,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B3,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.456</v>
+      </c>
+      <c r="Q4">
+        <f>(1+ VLOOKUP($C3,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.1280000000000001</v>
-      </c>
-      <c r="Q4">
-        <f>(1+ VLOOKUP($C4,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -16468,12 +16592,12 @@
         <v>2.25</v>
       </c>
       <c r="P5">
-        <f>(1+ VLOOKUP($B5,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B4,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1280000000000001</v>
+      </c>
+      <c r="Q5">
+        <f>(1+ VLOOKUP($C4,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.1080000000000001</v>
-      </c>
-      <c r="Q5">
-        <f>(1+ VLOOKUP($C5,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1280000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -16505,15 +16629,15 @@
       </c>
       <c r="M6">
         <f t="shared" si="1"/>
-        <v>2.2400000000000002</v>
+        <v>2.25</v>
       </c>
       <c r="P6">
-        <f>(1+ VLOOKUP($B6,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.121</v>
+        <f>(1+ VLOOKUP($B5,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
       </c>
       <c r="Q6">
-        <f>(1+ VLOOKUP($C6,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
+        <f>(1+ VLOOKUP($C5,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1280000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -16548,12 +16672,12 @@
         <v>2.2400000000000002</v>
       </c>
       <c r="P7">
-        <f>(1+ VLOOKUP($B7,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B6,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.121</v>
+      </c>
+      <c r="Q7">
+        <f>(1+ VLOOKUP($C6,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.1080000000000001</v>
-      </c>
-      <c r="Q7">
-        <f>(1+ VLOOKUP($C7,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.121</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -16585,15 +16709,15 @@
       </c>
       <c r="M8">
         <f t="shared" si="1"/>
-        <v>2.1799999999999997</v>
+        <v>2.2400000000000002</v>
       </c>
       <c r="P8">
-        <f>(1+ VLOOKUP($B8,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B7,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
+      </c>
+      <c r="Q8">
+        <f>(1+ VLOOKUP($C7,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.121</v>
-      </c>
-      <c r="Q8">
-        <f>(1+ VLOOKUP($C8,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.054</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -16628,12 +16752,12 @@
         <v>2.1799999999999997</v>
       </c>
       <c r="P9">
-        <f>(1+ VLOOKUP($B9,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B8,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.121</v>
+      </c>
+      <c r="Q9">
+        <f>(1+ VLOOKUP($C8,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.054</v>
-      </c>
-      <c r="Q9">
-        <f>(1+ VLOOKUP($C9,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.121</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -16665,15 +16789,15 @@
       </c>
       <c r="M10">
         <f t="shared" si="1"/>
-        <v>2.3200000000000003</v>
+        <v>2.1799999999999997</v>
       </c>
       <c r="P10">
-        <f>(1+ VLOOKUP($B10,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B9,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.054</v>
+      </c>
+      <c r="Q10">
+        <f>(1+ VLOOKUP($C9,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.121</v>
-      </c>
-      <c r="Q10">
-        <f>(1+ VLOOKUP($C10,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.18</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -16708,12 +16832,12 @@
         <v>2.3200000000000003</v>
       </c>
       <c r="P11">
-        <f>(1+ VLOOKUP($B11,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B10,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.121</v>
+      </c>
+      <c r="Q11">
+        <f>(1+ VLOOKUP($C10,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.18</v>
-      </c>
-      <c r="Q11">
-        <f>(1+ VLOOKUP($C11,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.121</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -16745,15 +16869,15 @@
       </c>
       <c r="M12">
         <f t="shared" si="1"/>
-        <v>2.31</v>
+        <v>2.3200000000000003</v>
       </c>
       <c r="P12">
-        <f>(1+ VLOOKUP($B12,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B11,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.18</v>
+      </c>
+      <c r="Q12">
+        <f>(1+ VLOOKUP($C11,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.121</v>
-      </c>
-      <c r="Q12">
-        <f>(1+ VLOOKUP($C12,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.165</v>
       </c>
     </row>
     <row r="13" spans="1:17">
@@ -16788,12 +16912,12 @@
         <v>2.31</v>
       </c>
       <c r="P13">
-        <f>(1+ VLOOKUP($B13,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B12,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.121</v>
+      </c>
+      <c r="Q13">
+        <f>(1+ VLOOKUP($C12,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.165</v>
-      </c>
-      <c r="Q13">
-        <f>(1+ VLOOKUP($C13,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.121</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -16825,15 +16949,15 @@
       </c>
       <c r="M14">
         <f t="shared" si="1"/>
-        <v>2.6100000000000003</v>
+        <v>2.31</v>
       </c>
       <c r="P14">
-        <f>(1+ VLOOKUP($B14,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.456</v>
+        <f>(1+ VLOOKUP($B13,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.165</v>
       </c>
       <c r="Q14">
-        <f>(1+ VLOOKUP($C14,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
+        <f>(1+ VLOOKUP($C13,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.121</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -16868,12 +16992,12 @@
         <v>2.6100000000000003</v>
       </c>
       <c r="P15">
-        <f>(1+ VLOOKUP($B15,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B14,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.456</v>
+      </c>
+      <c r="Q15">
+        <f>(1+ VLOOKUP($C14,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.1080000000000001</v>
-      </c>
-      <c r="Q15">
-        <f>(1+ VLOOKUP($C15,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.456</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -16905,15 +17029,15 @@
       </c>
       <c r="M16">
         <f t="shared" si="1"/>
-        <v>2.5300000000000002</v>
+        <v>2.6100000000000003</v>
       </c>
       <c r="P16">
-        <f>(1+ VLOOKUP($B16,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B15,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
+      </c>
+      <c r="Q16">
+        <f>(1+ VLOOKUP($C15,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.456</v>
-      </c>
-      <c r="Q16">
-        <f>(1+ VLOOKUP($C16,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.054</v>
       </c>
     </row>
     <row r="17" spans="1:17">
@@ -16948,12 +17072,12 @@
         <v>2.5300000000000002</v>
       </c>
       <c r="P17">
-        <f>(1+ VLOOKUP($B17,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B16,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.456</v>
+      </c>
+      <c r="Q17">
+        <f>(1+ VLOOKUP($C16,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.054</v>
-      </c>
-      <c r="Q17">
-        <f>(1+ VLOOKUP($C17,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.456</v>
       </c>
     </row>
     <row r="18" spans="1:17">
@@ -16985,15 +17109,15 @@
       </c>
       <c r="M18">
         <f t="shared" si="1"/>
-        <v>2.3899999999999997</v>
+        <v>2.5300000000000002</v>
       </c>
       <c r="P18">
-        <f>(1+ VLOOKUP($B18,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
+        <f>(1+ VLOOKUP($B17,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.054</v>
       </c>
       <c r="Q18">
-        <f>(1+ VLOOKUP($C18,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.25</v>
+        <f>(1+ VLOOKUP($C17,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.456</v>
       </c>
     </row>
     <row r="19" spans="1:17">
@@ -17028,12 +17152,12 @@
         <v>2.3899999999999997</v>
       </c>
       <c r="P19">
-        <f>(1+ VLOOKUP($B19,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B18,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
+      </c>
+      <c r="Q19">
+        <f>(1+ VLOOKUP($C18,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.25</v>
-      </c>
-      <c r="Q19">
-        <f>(1+ VLOOKUP($C19,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:17">
@@ -17065,15 +17189,15 @@
       </c>
       <c r="M20">
         <f t="shared" si="1"/>
-        <v>2.37</v>
+        <v>2.3899999999999997</v>
       </c>
       <c r="P20">
-        <f>(1+ VLOOKUP($B20,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B19,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.25</v>
+      </c>
+      <c r="Q20">
+        <f>(1+ VLOOKUP($C19,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.1080000000000001</v>
-      </c>
-      <c r="Q20">
-        <f>(1+ VLOOKUP($C20,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.238</v>
       </c>
     </row>
     <row r="21" spans="1:17">
@@ -17108,12 +17232,12 @@
         <v>2.37</v>
       </c>
       <c r="P21">
-        <f>(1+ VLOOKUP($B21,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B20,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
+      </c>
+      <c r="Q21">
+        <f>(1+ VLOOKUP($C20,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.238</v>
-      </c>
-      <c r="Q21">
-        <f>(1+ VLOOKUP($C21,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
       </c>
     </row>
     <row r="22" spans="1:17">
@@ -17145,15 +17269,15 @@
       </c>
       <c r="M22">
         <f t="shared" si="1"/>
-        <v>2.17</v>
+        <v>2.37</v>
       </c>
       <c r="P22">
-        <f>(1+ VLOOKUP($B22,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B21,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.238</v>
+      </c>
+      <c r="Q22">
+        <f>(1+ VLOOKUP($C21,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.1080000000000001</v>
-      </c>
-      <c r="Q22">
-        <f>(1+ VLOOKUP($C22,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.054</v>
       </c>
     </row>
     <row r="23" spans="1:17">
@@ -17188,12 +17312,12 @@
         <v>2.17</v>
       </c>
       <c r="P23">
-        <f>(1+ VLOOKUP($B23,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B22,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
+      </c>
+      <c r="Q23">
+        <f>(1+ VLOOKUP($C22,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.054</v>
-      </c>
-      <c r="Q23">
-        <f>(1+ VLOOKUP($C23,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
       </c>
     </row>
     <row r="24" spans="1:17">
@@ -17225,15 +17349,15 @@
       </c>
       <c r="M24">
         <f t="shared" si="1"/>
-        <v>2.31</v>
+        <v>2.17</v>
       </c>
       <c r="P24">
-        <f>(1+ VLOOKUP($B24,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B23,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.054</v>
+      </c>
+      <c r="Q24">
+        <f>(1+ VLOOKUP($C23,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.1080000000000001</v>
-      </c>
-      <c r="Q24">
-        <f>(1+ VLOOKUP($C24,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.18</v>
       </c>
     </row>
     <row r="25" spans="1:17">
@@ -17268,12 +17392,12 @@
         <v>2.31</v>
       </c>
       <c r="P25">
-        <f>(1+ VLOOKUP($B25,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B24,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
+      </c>
+      <c r="Q25">
+        <f>(1+ VLOOKUP($C24,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.18</v>
-      </c>
-      <c r="Q25">
-        <f>(1+ VLOOKUP($C25,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
       </c>
     </row>
     <row r="26" spans="1:17">
@@ -17305,15 +17429,15 @@
       </c>
       <c r="M26">
         <f t="shared" si="1"/>
-        <v>2.44</v>
+        <v>2.31</v>
       </c>
       <c r="P26">
-        <f>(1+ VLOOKUP($B26,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B25,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.18</v>
+      </c>
+      <c r="Q26">
+        <f>(1+ VLOOKUP($C25,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.1080000000000001</v>
-      </c>
-      <c r="Q26">
-        <f>(1+ VLOOKUP($C26,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.296</v>
       </c>
     </row>
     <row r="27" spans="1:17">
@@ -17348,12 +17472,12 @@
         <v>2.44</v>
       </c>
       <c r="P27">
-        <f>(1+ VLOOKUP($B27,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B26,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
+      </c>
+      <c r="Q27">
+        <f>(1+ VLOOKUP($C26,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.296</v>
-      </c>
-      <c r="Q27">
-        <f>(1+ VLOOKUP($C27,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:17">
@@ -17385,15 +17509,15 @@
       </c>
       <c r="M28">
         <f t="shared" si="1"/>
-        <v>1.76</v>
+        <v>2.44</v>
       </c>
       <c r="P28">
-        <f>(1+ VLOOKUP($B28,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B27,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.296</v>
+      </c>
+      <c r="Q28">
+        <f>(1+ VLOOKUP($C27,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.1080000000000001</v>
-      </c>
-      <c r="Q28">
-        <f>(1+ VLOOKUP($C28,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>0.69</v>
       </c>
     </row>
     <row r="29" spans="1:17">
@@ -17428,12 +17552,12 @@
         <v>1.76</v>
       </c>
       <c r="P29">
-        <f>(1+ VLOOKUP($B29,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B28,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
+      </c>
+      <c r="Q29">
+        <f>(1+ VLOOKUP($C28,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>0.69</v>
-      </c>
-      <c r="Q29">
-        <f>(1+ VLOOKUP($C29,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
       </c>
     </row>
     <row r="30" spans="1:17">
@@ -17465,15 +17589,15 @@
       </c>
       <c r="M30">
         <f t="shared" si="1"/>
-        <v>2.2800000000000002</v>
+        <v>1.76</v>
       </c>
       <c r="P30">
-        <f>(1+ VLOOKUP($B30,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B29,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>0.69</v>
+      </c>
+      <c r="Q30">
+        <f>(1+ VLOOKUP($C29,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.1080000000000001</v>
-      </c>
-      <c r="Q30">
-        <f>(1+ VLOOKUP($C30,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.157</v>
       </c>
     </row>
     <row r="31" spans="1:17">
@@ -17508,12 +17632,12 @@
         <v>2.2800000000000002</v>
       </c>
       <c r="P31">
-        <f>(1+ VLOOKUP($B31,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B30,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
+      </c>
+      <c r="Q31">
+        <f>(1+ VLOOKUP($C30,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.157</v>
-      </c>
-      <c r="Q31">
-        <f>(1+ VLOOKUP($C31,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
       </c>
     </row>
     <row r="32" spans="1:17">
@@ -17545,15 +17669,15 @@
       </c>
       <c r="M32">
         <f t="shared" si="1"/>
-        <v>2.29</v>
+        <v>2.2800000000000002</v>
       </c>
       <c r="P32">
-        <f>(1+ VLOOKUP($B32,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B31,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.157</v>
+      </c>
+      <c r="Q32">
+        <f>(1+ VLOOKUP($C31,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.1080000000000001</v>
-      </c>
-      <c r="Q32">
-        <f>(1+ VLOOKUP($C32,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.165</v>
       </c>
     </row>
     <row r="33" spans="1:17">
@@ -17588,12 +17712,12 @@
         <v>2.29</v>
       </c>
       <c r="P33">
-        <f>(1+ VLOOKUP($B33,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B32,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
+      </c>
+      <c r="Q33">
+        <f>(1+ VLOOKUP($C32,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.165</v>
-      </c>
-      <c r="Q33">
-        <f>(1+ VLOOKUP($C33,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
       </c>
     </row>
     <row r="34" spans="1:17">
@@ -17625,15 +17749,15 @@
       </c>
       <c r="M34">
         <f t="shared" si="1"/>
-        <v>2.5499999999999998</v>
+        <v>2.29</v>
       </c>
       <c r="P34">
-        <f>(1+ VLOOKUP($B34,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.25</v>
+        <f>(1+ VLOOKUP($B33,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.165</v>
       </c>
       <c r="Q34">
-        <f>(1+ VLOOKUP($C34,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.238</v>
+        <f>(1+ VLOOKUP($C33,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
       </c>
     </row>
     <row r="35" spans="1:17">
@@ -17668,12 +17792,12 @@
         <v>2.5499999999999998</v>
       </c>
       <c r="P35">
-        <f>(1+ VLOOKUP($B35,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B34,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.25</v>
+      </c>
+      <c r="Q35">
+        <f>(1+ VLOOKUP($C34,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.238</v>
-      </c>
-      <c r="Q35">
-        <f>(1+ VLOOKUP($C35,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.25</v>
       </c>
     </row>
     <row r="36" spans="1:17">
@@ -17705,15 +17829,15 @@
       </c>
       <c r="M36">
         <f t="shared" si="1"/>
-        <v>1.8599999999999999</v>
+        <v>2.5499999999999998</v>
       </c>
       <c r="P36">
-        <f>(1+ VLOOKUP($B36,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B35,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.238</v>
+      </c>
+      <c r="Q36">
+        <f>(1+ VLOOKUP($C35,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.25</v>
-      </c>
-      <c r="Q36">
-        <f>(1+ VLOOKUP($C36,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>0.69</v>
       </c>
     </row>
     <row r="37" spans="1:17">
@@ -17748,12 +17872,12 @@
         <v>1.8599999999999999</v>
       </c>
       <c r="P37">
-        <f>(1+ VLOOKUP($B37,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B36,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.25</v>
+      </c>
+      <c r="Q37">
+        <f>(1+ VLOOKUP($C36,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>0.69</v>
-      </c>
-      <c r="Q37">
-        <f>(1+ VLOOKUP($C37,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.25</v>
       </c>
     </row>
     <row r="38" spans="1:17">
@@ -17785,15 +17909,15 @@
       </c>
       <c r="M38">
         <f t="shared" si="1"/>
-        <v>2.4500000000000002</v>
+        <v>1.8599999999999999</v>
       </c>
       <c r="P38">
-        <f>(1+ VLOOKUP($B38,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B37,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>0.69</v>
+      </c>
+      <c r="Q38">
+        <f>(1+ VLOOKUP($C37,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.25</v>
-      </c>
-      <c r="Q38">
-        <f>(1+ VLOOKUP($C38,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.157</v>
       </c>
     </row>
     <row r="39" spans="1:17">
@@ -17828,12 +17952,12 @@
         <v>2.4500000000000002</v>
       </c>
       <c r="P39">
-        <f>(1+ VLOOKUP($B39,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B38,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.25</v>
+      </c>
+      <c r="Q39">
+        <f>(1+ VLOOKUP($C38,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.157</v>
-      </c>
-      <c r="Q39">
-        <f>(1+ VLOOKUP($C39,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.25</v>
       </c>
     </row>
     <row r="40" spans="1:17">
@@ -17865,15 +17989,15 @@
       </c>
       <c r="M40">
         <f t="shared" si="1"/>
-        <v>2.46</v>
+        <v>2.4500000000000002</v>
       </c>
       <c r="P40">
-        <f>(1+ VLOOKUP($B40,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.238</v>
+        <f>(1+ VLOOKUP($B39,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.157</v>
       </c>
       <c r="Q40">
-        <f>(1+ VLOOKUP($C40,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.18</v>
+        <f>(1+ VLOOKUP($C39,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.25</v>
       </c>
     </row>
     <row r="41" spans="1:17">
@@ -17908,12 +18032,12 @@
         <v>2.46</v>
       </c>
       <c r="P41">
-        <f>(1+ VLOOKUP($B41,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B40,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.238</v>
+      </c>
+      <c r="Q41">
+        <f>(1+ VLOOKUP($C40,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.18</v>
-      </c>
-      <c r="Q41">
-        <f>(1+ VLOOKUP($C41,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.238</v>
       </c>
     </row>
     <row r="42" spans="1:17">
@@ -17945,15 +18069,15 @@
       </c>
       <c r="M42">
         <f t="shared" si="1"/>
-        <v>2.6</v>
+        <v>2.46</v>
       </c>
       <c r="P42">
-        <f>(1+ VLOOKUP($B42,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B41,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.18</v>
+      </c>
+      <c r="Q42">
+        <f>(1+ VLOOKUP($C41,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.238</v>
-      </c>
-      <c r="Q42">
-        <f>(1+ VLOOKUP($C42,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.296</v>
       </c>
     </row>
     <row r="43" spans="1:17">
@@ -17988,12 +18112,12 @@
         <v>2.6</v>
       </c>
       <c r="P43">
-        <f>(1+ VLOOKUP($B43,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B42,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.238</v>
+      </c>
+      <c r="Q43">
+        <f>(1+ VLOOKUP($C42,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.296</v>
-      </c>
-      <c r="Q43">
-        <f>(1+ VLOOKUP($C43,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.238</v>
       </c>
     </row>
     <row r="44" spans="1:17">
@@ -18025,15 +18149,15 @@
       </c>
       <c r="M44">
         <f t="shared" si="1"/>
-        <v>2.44</v>
+        <v>2.6</v>
       </c>
       <c r="P44">
-        <f>(1+ VLOOKUP($B44,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B43,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.296</v>
+      </c>
+      <c r="Q44">
+        <f>(1+ VLOOKUP($C43,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.238</v>
-      </c>
-      <c r="Q44">
-        <f>(1+ VLOOKUP($C44,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.165</v>
       </c>
     </row>
     <row r="45" spans="1:17">
@@ -18068,12 +18192,12 @@
         <v>2.44</v>
       </c>
       <c r="P45">
-        <f>(1+ VLOOKUP($B45,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B44,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.238</v>
+      </c>
+      <c r="Q45">
+        <f>(1+ VLOOKUP($C44,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.165</v>
-      </c>
-      <c r="Q45">
-        <f>(1+ VLOOKUP($C45,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.238</v>
       </c>
     </row>
     <row r="46" spans="1:17">
@@ -18108,12 +18232,12 @@
         <v>2.44</v>
       </c>
       <c r="P46">
-        <f>(1+ VLOOKUP($B46,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B45,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.165</v>
+      </c>
+      <c r="Q46">
+        <f>(1+ VLOOKUP($C45,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.238</v>
-      </c>
-      <c r="Q46">
-        <f>(1+ VLOOKUP($C46,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.165</v>
       </c>
     </row>
     <row r="47" spans="1:17">
@@ -18148,12 +18272,12 @@
         <v>2.44</v>
       </c>
       <c r="P47">
-        <f>(1+ VLOOKUP($B47,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B46,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.238</v>
+      </c>
+      <c r="Q47">
+        <f>(1+ VLOOKUP($C46,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.165</v>
-      </c>
-      <c r="Q47">
-        <f>(1+ VLOOKUP($C47,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.238</v>
       </c>
     </row>
     <row r="48" spans="1:17">
@@ -18185,15 +18309,15 @@
       </c>
       <c r="M48">
         <f t="shared" si="1"/>
-        <v>1.88</v>
+        <v>2.44</v>
       </c>
       <c r="P48">
-        <f>(1+ VLOOKUP($B48,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>0.79600000000000004</v>
+        <f>(1+ VLOOKUP($B47,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.165</v>
       </c>
       <c r="Q48">
-        <f>(1+ VLOOKUP($C48,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
+        <f>(1+ VLOOKUP($C47,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.238</v>
       </c>
     </row>
     <row r="49" spans="1:17">
@@ -18228,12 +18352,12 @@
         <v>1.88</v>
       </c>
       <c r="P49">
-        <f>(1+ VLOOKUP($B49,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B48,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>0.79600000000000004</v>
+      </c>
+      <c r="Q49">
+        <f>(1+ VLOOKUP($C48,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.1080000000000001</v>
-      </c>
-      <c r="Q49">
-        <f>(1+ VLOOKUP($C49,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>0.79600000000000004</v>
       </c>
     </row>
     <row r="50" spans="1:17">
@@ -18265,15 +18389,15 @@
       </c>
       <c r="M50">
         <f t="shared" si="1"/>
-        <v>1.56</v>
+        <v>1.88</v>
       </c>
       <c r="P50">
-        <f>(1+ VLOOKUP($B50,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B49,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
+      </c>
+      <c r="Q50">
+        <f>(1+ VLOOKUP($C49,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>0.79600000000000004</v>
-      </c>
-      <c r="Q50">
-        <f>(1+ VLOOKUP($C50,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>0.70100000000000007</v>
       </c>
     </row>
     <row r="51" spans="1:17">
@@ -18308,12 +18432,12 @@
         <v>1.56</v>
       </c>
       <c r="P51">
-        <f>(1+ VLOOKUP($B51,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B50,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>0.79600000000000004</v>
+      </c>
+      <c r="Q51">
+        <f>(1+ VLOOKUP($C50,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>0.70100000000000007</v>
-      </c>
-      <c r="Q51">
-        <f>(1+ VLOOKUP($C51,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>0.79600000000000004</v>
       </c>
     </row>
     <row r="52" spans="1:17">
@@ -18345,15 +18469,15 @@
       </c>
       <c r="M52">
         <f t="shared" si="1"/>
-        <v>1.97</v>
+        <v>1.56</v>
       </c>
       <c r="P52">
-        <f>(1+ VLOOKUP($B52,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>0.91700000000000004</v>
+        <f>(1+ VLOOKUP($B51,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>0.70100000000000007</v>
       </c>
       <c r="Q52">
-        <f>(1+ VLOOKUP($C52,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.054</v>
+        <f>(1+ VLOOKUP($C51,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>0.79600000000000004</v>
       </c>
     </row>
     <row r="53" spans="1:17">
@@ -18388,12 +18512,12 @@
         <v>1.97</v>
       </c>
       <c r="P53">
-        <f>(1+ VLOOKUP($B53,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B52,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>0.91700000000000004</v>
+      </c>
+      <c r="Q53">
+        <f>(1+ VLOOKUP($C52,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.054</v>
-      </c>
-      <c r="Q53">
-        <f>(1+ VLOOKUP($C53,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>0.91700000000000004</v>
       </c>
     </row>
     <row r="54" spans="1:17">
@@ -18425,15 +18549,15 @@
       </c>
       <c r="M54">
         <f t="shared" si="1"/>
-        <v>2.4699999999999998</v>
+        <v>1.97</v>
       </c>
       <c r="P54">
-        <f>(1+ VLOOKUP($B54,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
+        <f>(1+ VLOOKUP($B53,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.054</v>
       </c>
       <c r="Q54">
-        <f>(1+ VLOOKUP($C54,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.325</v>
+        <f>(1+ VLOOKUP($C53,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>0.91700000000000004</v>
       </c>
     </row>
     <row r="55" spans="1:17">
@@ -18468,12 +18592,12 @@
         <v>2.4699999999999998</v>
       </c>
       <c r="P55">
-        <f>(1+ VLOOKUP($B55,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B54,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
+      </c>
+      <c r="Q55">
+        <f>(1+ VLOOKUP($C54,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.325</v>
-      </c>
-      <c r="Q55">
-        <f>(1+ VLOOKUP($C55,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
       </c>
     </row>
     <row r="56" spans="1:17">
@@ -18505,15 +18629,15 @@
       </c>
       <c r="M56">
         <f t="shared" si="1"/>
-        <v>2.31</v>
+        <v>2.4699999999999998</v>
       </c>
       <c r="P56">
-        <f>(1+ VLOOKUP($B56,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B55,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.325</v>
+      </c>
+      <c r="Q56">
+        <f>(1+ VLOOKUP($C55,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.1080000000000001</v>
-      </c>
-      <c r="Q56">
-        <f>(1+ VLOOKUP($C56,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.181</v>
       </c>
     </row>
     <row r="57" spans="1:17">
@@ -18548,12 +18672,12 @@
         <v>2.31</v>
       </c>
       <c r="P57">
-        <f>(1+ VLOOKUP($B57,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B56,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
+      </c>
+      <c r="Q57">
+        <f>(1+ VLOOKUP($C56,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.181</v>
-      </c>
-      <c r="Q57">
-        <f>(1+ VLOOKUP($C57,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
       </c>
     </row>
     <row r="58" spans="1:17">
@@ -18585,15 +18709,15 @@
       </c>
       <c r="M58">
         <f t="shared" si="1"/>
-        <v>2.29</v>
+        <v>2.31</v>
       </c>
       <c r="P58">
-        <f>(1+ VLOOKUP($B58,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B57,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.181</v>
+      </c>
+      <c r="Q58">
+        <f>(1+ VLOOKUP($C57,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.1080000000000001</v>
-      </c>
-      <c r="Q58">
-        <f>(1+ VLOOKUP($C58,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.165</v>
       </c>
     </row>
     <row r="59" spans="1:17">
@@ -18628,12 +18752,12 @@
         <v>2.29</v>
       </c>
       <c r="P59">
-        <f>(1+ VLOOKUP($B59,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B58,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
+      </c>
+      <c r="Q59">
+        <f>(1+ VLOOKUP($C58,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.165</v>
-      </c>
-      <c r="Q59">
-        <f>(1+ VLOOKUP($C59,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.1080000000000001</v>
       </c>
     </row>
     <row r="60" spans="1:17">
@@ -18665,15 +18789,15 @@
       </c>
       <c r="M60">
         <f t="shared" si="1"/>
-        <v>2.23</v>
+        <v>2.29</v>
       </c>
       <c r="P60">
-        <f>(1+ VLOOKUP($B60,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.054</v>
+        <f>(1+ VLOOKUP($B59,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.165</v>
       </c>
       <c r="Q60">
-        <f>(1+ VLOOKUP($C60,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.165</v>
+        <f>(1+ VLOOKUP($C59,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.1080000000000001</v>
       </c>
     </row>
     <row r="61" spans="1:17">
@@ -18708,12 +18832,12 @@
         <v>2.23</v>
       </c>
       <c r="P61">
-        <f>(1+ VLOOKUP($B61,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B60,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.054</v>
+      </c>
+      <c r="Q61">
+        <f>(1+ VLOOKUP($C60,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.165</v>
-      </c>
-      <c r="Q61">
-        <f>(1+ VLOOKUP($C61,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.054</v>
       </c>
     </row>
     <row r="62" spans="1:17">
@@ -18745,15 +18869,15 @@
       </c>
       <c r="M62">
         <f t="shared" si="1"/>
-        <v>1.54</v>
+        <v>2.23</v>
       </c>
       <c r="P62">
-        <f>(1+ VLOOKUP($B62,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>0.76700000000000002</v>
+        <f>(1+ VLOOKUP($B61,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.165</v>
       </c>
       <c r="Q62">
-        <f>(1+ VLOOKUP($C62,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>0.70100000000000007</v>
+        <f>(1+ VLOOKUP($C61,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.054</v>
       </c>
     </row>
     <row r="63" spans="1:17">
@@ -18788,12 +18912,12 @@
         <v>1.54</v>
       </c>
       <c r="P63">
-        <f>(1+ VLOOKUP($B63,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B62,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>0.76700000000000002</v>
+      </c>
+      <c r="Q63">
+        <f>(1+ VLOOKUP($C62,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>0.70100000000000007</v>
-      </c>
-      <c r="Q63">
-        <f>(1+ VLOOKUP($C63,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>0.76700000000000002</v>
       </c>
     </row>
     <row r="64" spans="1:17">
@@ -18825,15 +18949,15 @@
       </c>
       <c r="M64">
         <f t="shared" si="1"/>
-        <v>1.53</v>
+        <v>1.54</v>
       </c>
       <c r="P64">
-        <f>(1+ VLOOKUP($B64,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B63,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>0.70100000000000007</v>
+      </c>
+      <c r="Q64">
+        <f>(1+ VLOOKUP($C63,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>0.76700000000000002</v>
-      </c>
-      <c r="Q64">
-        <f>(1+ VLOOKUP($C64,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>0.69</v>
       </c>
     </row>
     <row r="65" spans="1:17">
@@ -18868,12 +18992,12 @@
         <v>1.53</v>
       </c>
       <c r="P65">
-        <f>(1+ VLOOKUP($B65,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B64,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>0.76700000000000002</v>
+      </c>
+      <c r="Q65">
+        <f>(1+ VLOOKUP($C64,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>0.69</v>
-      </c>
-      <c r="Q65">
-        <f>(1+ VLOOKUP($C65,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>0.76700000000000002</v>
       </c>
     </row>
     <row r="66" spans="1:17">
@@ -18905,15 +19029,15 @@
       </c>
       <c r="M66">
         <f t="shared" si="1"/>
-        <v>1.8900000000000001</v>
+        <v>1.53</v>
       </c>
       <c r="P66">
-        <f>(1+ VLOOKUP($B66,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B65,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>0.69</v>
+      </c>
+      <c r="Q66">
+        <f>(1+ VLOOKUP($C65,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>0.76700000000000002</v>
-      </c>
-      <c r="Q66">
-        <f>(1+ VLOOKUP($C66,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.157</v>
       </c>
     </row>
     <row r="67" spans="1:17">
@@ -18936,7 +19060,7 @@
         <v>700</v>
       </c>
       <c r="G67" s="19">
-        <f t="shared" ref="G67:G93" si="2">M67</f>
+        <f t="shared" ref="G67:G93" si="2">M68</f>
         <v>1.8900000000000001</v>
       </c>
       <c r="I67" s="19" t="str">
@@ -18944,16 +19068,16 @@
         <v/>
       </c>
       <c r="M67">
-        <f t="shared" ref="M67:M93" si="3">ROUND(P67*Q67, 2)+1</f>
+        <f t="shared" si="1"/>
         <v>1.8900000000000001</v>
       </c>
       <c r="P67">
-        <f>(1+ VLOOKUP($B67,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B66,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>0.76700000000000002</v>
+      </c>
+      <c r="Q67">
+        <f>(1+ VLOOKUP($C66,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.157</v>
-      </c>
-      <c r="Q67">
-        <f>(1+ VLOOKUP($C67,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>0.76700000000000002</v>
       </c>
     </row>
     <row r="68" spans="1:17">
@@ -18984,16 +19108,16 @@
         <v/>
       </c>
       <c r="M68">
-        <f t="shared" si="3"/>
-        <v>2.5300000000000002</v>
+        <f t="shared" ref="M68:M94" si="3">ROUND(P68*Q68, 2)+1</f>
+        <v>1.8900000000000001</v>
       </c>
       <c r="P68">
-        <f>(1+ VLOOKUP($B68,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.18</v>
+        <f>(1+ VLOOKUP($B67,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.157</v>
       </c>
       <c r="Q68">
-        <f>(1+ VLOOKUP($C68,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.296</v>
+        <f>(1+ VLOOKUP($C67,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>0.76700000000000002</v>
       </c>
     </row>
     <row r="69" spans="1:17">
@@ -19028,12 +19152,12 @@
         <v>2.5300000000000002</v>
       </c>
       <c r="P69">
-        <f>(1+ VLOOKUP($B69,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B68,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.18</v>
+      </c>
+      <c r="Q69">
+        <f>(1+ VLOOKUP($C68,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.296</v>
-      </c>
-      <c r="Q69">
-        <f>(1+ VLOOKUP($C69,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.18</v>
       </c>
     </row>
     <row r="70" spans="1:17">
@@ -19065,15 +19189,15 @@
       </c>
       <c r="M70">
         <f t="shared" si="3"/>
-        <v>2.37</v>
+        <v>2.5300000000000002</v>
       </c>
       <c r="P70">
-        <f>(1+ VLOOKUP($B70,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B69,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.296</v>
+      </c>
+      <c r="Q70">
+        <f>(1+ VLOOKUP($C69,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.18</v>
-      </c>
-      <c r="Q70">
-        <f>(1+ VLOOKUP($C70,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.165</v>
       </c>
     </row>
     <row r="71" spans="1:17">
@@ -19108,12 +19232,12 @@
         <v>2.37</v>
       </c>
       <c r="P71">
-        <f>(1+ VLOOKUP($B71,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B70,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.18</v>
+      </c>
+      <c r="Q71">
+        <f>(1+ VLOOKUP($C70,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.165</v>
-      </c>
-      <c r="Q71">
-        <f>(1+ VLOOKUP($C71,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.18</v>
       </c>
     </row>
     <row r="72" spans="1:17">
@@ -19145,15 +19269,15 @@
       </c>
       <c r="M72">
         <f t="shared" si="3"/>
-        <v>2.74</v>
+        <v>2.37</v>
       </c>
       <c r="P72">
-        <f>(1+ VLOOKUP($B72,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.31</v>
+        <f>(1+ VLOOKUP($B71,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.165</v>
       </c>
       <c r="Q72">
-        <f>(1+ VLOOKUP($C72,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.325</v>
+        <f>(1+ VLOOKUP($C71,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.18</v>
       </c>
     </row>
     <row r="73" spans="1:17">
@@ -19188,12 +19312,12 @@
         <v>2.74</v>
       </c>
       <c r="P73">
-        <f>(1+ VLOOKUP($B73,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B72,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.31</v>
+      </c>
+      <c r="Q73">
+        <f>(1+ VLOOKUP($C72,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.325</v>
-      </c>
-      <c r="Q73">
-        <f>(1+ VLOOKUP($C73,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.31</v>
       </c>
     </row>
     <row r="74" spans="1:17">
@@ -19225,15 +19349,15 @@
       </c>
       <c r="M74">
         <f t="shared" si="3"/>
-        <v>2.7</v>
+        <v>2.74</v>
       </c>
       <c r="P74">
-        <f>(1+ VLOOKUP($B74,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B73,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.325</v>
+      </c>
+      <c r="Q74">
+        <f>(1+ VLOOKUP($C73,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.31</v>
-      </c>
-      <c r="Q74">
-        <f>(1+ VLOOKUP($C74,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.296</v>
       </c>
     </row>
     <row r="75" spans="1:17">
@@ -19268,12 +19392,12 @@
         <v>2.7</v>
       </c>
       <c r="P75">
-        <f>(1+ VLOOKUP($B75,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B74,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.31</v>
+      </c>
+      <c r="Q75">
+        <f>(1+ VLOOKUP($C74,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.296</v>
-      </c>
-      <c r="Q75">
-        <f>(1+ VLOOKUP($C75,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.31</v>
       </c>
     </row>
     <row r="76" spans="1:17">
@@ -19305,15 +19429,15 @@
       </c>
       <c r="M76">
         <f t="shared" si="3"/>
-        <v>2.54</v>
+        <v>2.7</v>
       </c>
       <c r="P76">
-        <f>(1+ VLOOKUP($B76,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B75,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.296</v>
+      </c>
+      <c r="Q76">
+        <f>(1+ VLOOKUP($C75,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.31</v>
-      </c>
-      <c r="Q76">
-        <f>(1+ VLOOKUP($C76,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.173</v>
       </c>
     </row>
     <row r="77" spans="1:17">
@@ -19348,12 +19472,12 @@
         <v>2.54</v>
       </c>
       <c r="P77">
-        <f>(1+ VLOOKUP($B77,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B76,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.31</v>
+      </c>
+      <c r="Q77">
+        <f>(1+ VLOOKUP($C76,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.173</v>
-      </c>
-      <c r="Q77">
-        <f>(1+ VLOOKUP($C77,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.31</v>
       </c>
     </row>
     <row r="78" spans="1:17">
@@ -19385,15 +19509,15 @@
       </c>
       <c r="M78">
         <f t="shared" si="3"/>
-        <v>2.56</v>
+        <v>2.54</v>
       </c>
       <c r="P78">
-        <f>(1+ VLOOKUP($B78,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.325</v>
+        <f>(1+ VLOOKUP($B77,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.173</v>
       </c>
       <c r="Q78">
-        <f>(1+ VLOOKUP($C78,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.181</v>
+        <f>(1+ VLOOKUP($C77,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.31</v>
       </c>
     </row>
     <row r="79" spans="1:17">
@@ -19428,12 +19552,12 @@
         <v>2.56</v>
       </c>
       <c r="P79">
-        <f>(1+ VLOOKUP($B79,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B78,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.325</v>
+      </c>
+      <c r="Q79">
+        <f>(1+ VLOOKUP($C78,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.181</v>
-      </c>
-      <c r="Q79">
-        <f>(1+ VLOOKUP($C79,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.325</v>
       </c>
     </row>
     <row r="80" spans="1:17">
@@ -19465,15 +19589,15 @@
       </c>
       <c r="M80">
         <f t="shared" si="3"/>
-        <v>2.5499999999999998</v>
+        <v>2.56</v>
       </c>
       <c r="P80">
-        <f>(1+ VLOOKUP($B80,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B79,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.181</v>
+      </c>
+      <c r="Q80">
+        <f>(1+ VLOOKUP($C79,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.325</v>
-      </c>
-      <c r="Q80">
-        <f>(1+ VLOOKUP($C80,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.173</v>
       </c>
     </row>
     <row r="81" spans="1:17">
@@ -19508,12 +19632,12 @@
         <v>2.5499999999999998</v>
       </c>
       <c r="P81">
-        <f>(1+ VLOOKUP($B81,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B80,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.325</v>
+      </c>
+      <c r="Q81">
+        <f>(1+ VLOOKUP($C80,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.173</v>
-      </c>
-      <c r="Q81">
-        <f>(1+ VLOOKUP($C81,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.325</v>
       </c>
     </row>
     <row r="82" spans="1:17">
@@ -19545,15 +19669,15 @@
       </c>
       <c r="M82">
         <f t="shared" si="3"/>
-        <v>2.5099999999999998</v>
+        <v>2.5499999999999998</v>
       </c>
       <c r="P82">
-        <f>(1+ VLOOKUP($B82,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.296</v>
+        <f>(1+ VLOOKUP($B81,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.173</v>
       </c>
       <c r="Q82">
-        <f>(1+ VLOOKUP($C82,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.165</v>
+        <f>(1+ VLOOKUP($C81,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.325</v>
       </c>
     </row>
     <row r="83" spans="1:17">
@@ -19588,12 +19712,12 @@
         <v>2.5099999999999998</v>
       </c>
       <c r="P83">
-        <f>(1+ VLOOKUP($B83,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B82,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.296</v>
+      </c>
+      <c r="Q83">
+        <f>(1+ VLOOKUP($C82,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.165</v>
-      </c>
-      <c r="Q83">
-        <f>(1+ VLOOKUP($C83,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.296</v>
       </c>
     </row>
     <row r="84" spans="1:17">
@@ -19628,12 +19752,12 @@
         <v>2.5099999999999998</v>
       </c>
       <c r="P84">
-        <f>(1+ VLOOKUP($B84,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B83,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.165</v>
+      </c>
+      <c r="Q84">
+        <f>(1+ VLOOKUP($C83,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.296</v>
-      </c>
-      <c r="Q84">
-        <f>(1+ VLOOKUP($C84,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.165</v>
       </c>
     </row>
     <row r="85" spans="1:17">
@@ -19668,12 +19792,12 @@
         <v>2.5099999999999998</v>
       </c>
       <c r="P85">
-        <f>(1+ VLOOKUP($B85,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B84,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.296</v>
+      </c>
+      <c r="Q85">
+        <f>(1+ VLOOKUP($C84,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.165</v>
-      </c>
-      <c r="Q85">
-        <f>(1+ VLOOKUP($C85,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.296</v>
       </c>
     </row>
     <row r="86" spans="1:17">
@@ -19705,15 +19829,15 @@
       </c>
       <c r="M86">
         <f t="shared" si="3"/>
-        <v>1.8</v>
+        <v>2.5099999999999998</v>
       </c>
       <c r="P86">
-        <f>(1+ VLOOKUP($B86,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>0.69</v>
+        <f>(1+ VLOOKUP($B85,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.165</v>
       </c>
       <c r="Q86">
-        <f>(1+ VLOOKUP($C86,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.157</v>
+        <f>(1+ VLOOKUP($C85,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.296</v>
       </c>
     </row>
     <row r="87" spans="1:17">
@@ -19748,12 +19872,12 @@
         <v>1.8</v>
       </c>
       <c r="P87">
-        <f>(1+ VLOOKUP($B87,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B86,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>0.69</v>
+      </c>
+      <c r="Q87">
+        <f>(1+ VLOOKUP($C86,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.157</v>
-      </c>
-      <c r="Q87">
-        <f>(1+ VLOOKUP($C87,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>0.69</v>
       </c>
     </row>
     <row r="88" spans="1:17">
@@ -19785,15 +19909,15 @@
       </c>
       <c r="M88">
         <f t="shared" si="3"/>
-        <v>2.3899999999999997</v>
+        <v>1.8</v>
       </c>
       <c r="P88">
-        <f>(1+ VLOOKUP($B88,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.181</v>
+        <f>(1+ VLOOKUP($B87,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.157</v>
       </c>
       <c r="Q88">
-        <f>(1+ VLOOKUP($C88,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.173</v>
+        <f>(1+ VLOOKUP($C87,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>0.69</v>
       </c>
     </row>
     <row r="89" spans="1:17">
@@ -19828,12 +19952,12 @@
         <v>2.3899999999999997</v>
       </c>
       <c r="P89">
-        <f>(1+ VLOOKUP($B89,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B88,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.181</v>
+      </c>
+      <c r="Q89">
+        <f>(1+ VLOOKUP($C88,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.173</v>
-      </c>
-      <c r="Q89">
-        <f>(1+ VLOOKUP($C89,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.181</v>
       </c>
     </row>
     <row r="90" spans="1:17">
@@ -19865,15 +19989,15 @@
       </c>
       <c r="M90">
         <f t="shared" si="3"/>
-        <v>2.37</v>
+        <v>2.3899999999999997</v>
       </c>
       <c r="P90">
-        <f>(1+ VLOOKUP($B90,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B89,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.173</v>
       </c>
       <c r="Q90">
-        <f>(1+ VLOOKUP($C90,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.165</v>
+        <f>(1+ VLOOKUP($C89,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.181</v>
       </c>
     </row>
     <row r="91" spans="1:17">
@@ -19908,12 +20032,12 @@
         <v>2.37</v>
       </c>
       <c r="P91">
-        <f>(1+ VLOOKUP($B91,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B90,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.173</v>
+      </c>
+      <c r="Q91">
+        <f>(1+ VLOOKUP($C90,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.165</v>
-      </c>
-      <c r="Q91">
-        <f>(1+ VLOOKUP($C91,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.173</v>
       </c>
     </row>
     <row r="92" spans="1:17">
@@ -19945,15 +20069,15 @@
       </c>
       <c r="M92">
         <f t="shared" si="3"/>
-        <v>2.35</v>
+        <v>2.37</v>
       </c>
       <c r="P92">
-        <f>(1+ VLOOKUP($B92,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <f>(1+ VLOOKUP($B91,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.165</v>
       </c>
       <c r="Q92">
-        <f>(1+ VLOOKUP($C92,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
-        <v>1.157</v>
+        <f>(1+ VLOOKUP($C91,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.173</v>
       </c>
     </row>
     <row r="93" spans="1:17">
@@ -19988,10 +20112,24 @@
         <v>2.35</v>
       </c>
       <c r="P93">
+        <f>(1+ VLOOKUP($B92,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.165</v>
+      </c>
+      <c r="Q93">
+        <f>(1+ VLOOKUP($C92,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
+        <v>1.157</v>
+      </c>
+    </row>
+    <row r="94" spans="1:17">
+      <c r="M94">
+        <f t="shared" si="3"/>
+        <v>2.35</v>
+      </c>
+      <c r="P94">
         <f>(1+ VLOOKUP($B93,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.157</v>
       </c>
-      <c r="Q93">
+      <c r="Q94">
         <f>(1+ VLOOKUP($C93,'vomcost mult'!$N$10:$R$32,5, FALSE))</f>
         <v>1.165</v>
       </c>
@@ -20095,7 +20233,7 @@
         <v>223</v>
       </c>
       <c r="G1" s="56" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -21424,38 +21562,38 @@
       </c>
     </row>
     <row r="3" spans="1:30" ht="15.75" thickBot="1">
-      <c r="A3" s="79" t="s">
+      <c r="A3" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="80"/>
-      <c r="C3" s="80"/>
-      <c r="D3" s="80"/>
-      <c r="E3" s="80"/>
-      <c r="F3" s="80"/>
-      <c r="G3" s="80"/>
-      <c r="H3" s="80"/>
-      <c r="I3" s="80"/>
-      <c r="J3" s="80"/>
-      <c r="K3" s="80"/>
-      <c r="L3" s="80"/>
-      <c r="M3" s="80"/>
-      <c r="N3" s="80"/>
-      <c r="O3" s="80"/>
-      <c r="P3" s="80"/>
-      <c r="Q3" s="80"/>
-      <c r="R3" s="80"/>
-      <c r="S3" s="80"/>
-      <c r="T3" s="80"/>
-      <c r="U3" s="80"/>
-      <c r="V3" s="80"/>
-      <c r="W3" s="80"/>
-      <c r="X3" s="80"/>
-      <c r="Y3" s="80"/>
-      <c r="Z3" s="80"/>
-      <c r="AA3" s="80"/>
-      <c r="AB3" s="80"/>
-      <c r="AC3" s="80"/>
-      <c r="AD3" s="80"/>
+      <c r="B3" s="83"/>
+      <c r="C3" s="83"/>
+      <c r="D3" s="83"/>
+      <c r="E3" s="83"/>
+      <c r="F3" s="83"/>
+      <c r="G3" s="83"/>
+      <c r="H3" s="83"/>
+      <c r="I3" s="83"/>
+      <c r="J3" s="83"/>
+      <c r="K3" s="83"/>
+      <c r="L3" s="83"/>
+      <c r="M3" s="83"/>
+      <c r="N3" s="83"/>
+      <c r="O3" s="83"/>
+      <c r="P3" s="83"/>
+      <c r="Q3" s="83"/>
+      <c r="R3" s="83"/>
+      <c r="S3" s="83"/>
+      <c r="T3" s="83"/>
+      <c r="U3" s="83"/>
+      <c r="V3" s="83"/>
+      <c r="W3" s="83"/>
+      <c r="X3" s="83"/>
+      <c r="Y3" s="83"/>
+      <c r="Z3" s="83"/>
+      <c r="AA3" s="83"/>
+      <c r="AB3" s="83"/>
+      <c r="AC3" s="83"/>
+      <c r="AD3" s="83"/>
     </row>
     <row r="4" spans="1:30" ht="16.5" thickBot="1">
       <c r="A4" s="2" t="s">
@@ -21548,38 +21686,38 @@
       </c>
     </row>
     <row r="5" spans="1:30" ht="16.5" thickBot="1">
-      <c r="A5" s="81" t="s">
+      <c r="A5" s="84" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="82"/>
-      <c r="C5" s="82"/>
-      <c r="D5" s="82"/>
-      <c r="E5" s="82"/>
-      <c r="F5" s="82"/>
-      <c r="G5" s="82"/>
-      <c r="H5" s="82"/>
-      <c r="I5" s="82"/>
-      <c r="J5" s="82"/>
-      <c r="K5" s="82"/>
-      <c r="L5" s="82"/>
-      <c r="M5" s="82"/>
-      <c r="N5" s="82"/>
-      <c r="O5" s="82"/>
-      <c r="P5" s="82"/>
-      <c r="Q5" s="82"/>
-      <c r="R5" s="82"/>
-      <c r="S5" s="82"/>
-      <c r="T5" s="82"/>
-      <c r="U5" s="82"/>
-      <c r="V5" s="82"/>
-      <c r="W5" s="82"/>
-      <c r="X5" s="82"/>
-      <c r="Y5" s="82"/>
-      <c r="Z5" s="82"/>
-      <c r="AA5" s="82"/>
-      <c r="AB5" s="82"/>
-      <c r="AC5" s="82"/>
-      <c r="AD5" s="83"/>
+      <c r="B5" s="85"/>
+      <c r="C5" s="85"/>
+      <c r="D5" s="85"/>
+      <c r="E5" s="85"/>
+      <c r="F5" s="85"/>
+      <c r="G5" s="85"/>
+      <c r="H5" s="85"/>
+      <c r="I5" s="85"/>
+      <c r="J5" s="85"/>
+      <c r="K5" s="85"/>
+      <c r="L5" s="85"/>
+      <c r="M5" s="85"/>
+      <c r="N5" s="85"/>
+      <c r="O5" s="85"/>
+      <c r="P5" s="85"/>
+      <c r="Q5" s="85"/>
+      <c r="R5" s="85"/>
+      <c r="S5" s="85"/>
+      <c r="T5" s="85"/>
+      <c r="U5" s="85"/>
+      <c r="V5" s="85"/>
+      <c r="W5" s="85"/>
+      <c r="X5" s="85"/>
+      <c r="Y5" s="85"/>
+      <c r="Z5" s="85"/>
+      <c r="AA5" s="85"/>
+      <c r="AB5" s="85"/>
+      <c r="AC5" s="85"/>
+      <c r="AD5" s="86"/>
     </row>
     <row r="6" spans="1:30" ht="16.5" thickBot="1">
       <c r="A6" s="4"/>
@@ -34331,31 +34469,31 @@
     </row>
     <row r="2" spans="2:24" ht="15.75" thickBot="1"/>
     <row r="3" spans="2:24" ht="16.5" thickBot="1">
-      <c r="B3" s="84" t="s">
+      <c r="B3" s="87" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="85"/>
-      <c r="D3" s="85"/>
-      <c r="E3" s="85"/>
-      <c r="F3" s="85"/>
-      <c r="G3" s="85"/>
-      <c r="H3" s="85"/>
-      <c r="I3" s="85"/>
-      <c r="J3" s="85"/>
-      <c r="K3" s="85"/>
-      <c r="L3" s="85"/>
-      <c r="M3" s="85"/>
-      <c r="N3" s="85"/>
-      <c r="O3" s="85"/>
-      <c r="P3" s="85"/>
-      <c r="Q3" s="85"/>
-      <c r="R3" s="85"/>
-      <c r="S3" s="85"/>
-      <c r="T3" s="85"/>
-      <c r="U3" s="85"/>
-      <c r="V3" s="85"/>
-      <c r="W3" s="85"/>
-      <c r="X3" s="86"/>
+      <c r="C3" s="88"/>
+      <c r="D3" s="88"/>
+      <c r="E3" s="88"/>
+      <c r="F3" s="88"/>
+      <c r="G3" s="88"/>
+      <c r="H3" s="88"/>
+      <c r="I3" s="88"/>
+      <c r="J3" s="88"/>
+      <c r="K3" s="88"/>
+      <c r="L3" s="88"/>
+      <c r="M3" s="88"/>
+      <c r="N3" s="88"/>
+      <c r="O3" s="88"/>
+      <c r="P3" s="88"/>
+      <c r="Q3" s="88"/>
+      <c r="R3" s="88"/>
+      <c r="S3" s="88"/>
+      <c r="T3" s="88"/>
+      <c r="U3" s="88"/>
+      <c r="V3" s="88"/>
+      <c r="W3" s="88"/>
+      <c r="X3" s="89"/>
     </row>
     <row r="4" spans="2:24" ht="23.25" thickBot="1">
       <c r="B4" s="12" t="s">
@@ -36528,10 +36666,10 @@
       </c>
     </row>
     <row r="33" spans="1:24" ht="16.5" thickBot="1">
-      <c r="B33" s="87" t="s">
+      <c r="B33" s="90" t="s">
         <v>57</v>
       </c>
-      <c r="C33" s="88"/>
+      <c r="C33" s="91"/>
       <c r="D33" s="16"/>
       <c r="E33" s="16"/>
       <c r="F33" s="16"/>
@@ -40418,7 +40556,7 @@
         <v>111</v>
       </c>
       <c r="C25" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D25">
         <f t="shared" ref="D25:S40" ca="1" si="6">SUMIFS( INDIRECT(CONCATENATE($C25,"!", $A25, ":", $A25)),  INDIRECT(CONCATENATE($C25, "!$4:$4")), D$1)</f>
@@ -40538,7 +40676,7 @@
         <v>114</v>
       </c>
       <c r="C26" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D26">
         <f t="shared" ca="1" si="6"/>
@@ -40658,7 +40796,7 @@
         <v>116</v>
       </c>
       <c r="C27" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D27">
         <f t="shared" ca="1" si="6"/>
@@ -40778,7 +40916,7 @@
         <v>117</v>
       </c>
       <c r="C28" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D28">
         <f t="shared" ca="1" si="6"/>
@@ -40898,7 +41036,7 @@
         <v>118</v>
       </c>
       <c r="C29" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D29">
         <f t="shared" ca="1" si="6"/>
@@ -41018,7 +41156,7 @@
         <v>119</v>
       </c>
       <c r="C30" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D30">
         <f t="shared" ca="1" si="6"/>
@@ -41138,7 +41276,7 @@
         <v>120</v>
       </c>
       <c r="C31" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D31">
         <f t="shared" ca="1" si="6"/>
@@ -41258,7 +41396,7 @@
         <v>121</v>
       </c>
       <c r="C32" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D32">
         <f t="shared" ca="1" si="6"/>
@@ -41378,7 +41516,7 @@
         <v>122</v>
       </c>
       <c r="C33" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D33">
         <f t="shared" ca="1" si="6"/>
@@ -41498,7 +41636,7 @@
         <v>123</v>
       </c>
       <c r="C34" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D34">
         <f t="shared" ca="1" si="6"/>
@@ -41618,7 +41756,7 @@
         <v>124</v>
       </c>
       <c r="C35" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D35">
         <f t="shared" ca="1" si="6"/>
@@ -41738,7 +41876,7 @@
         <v>125</v>
       </c>
       <c r="C36" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D36">
         <f t="shared" ca="1" si="6"/>
@@ -41858,7 +41996,7 @@
         <v>126</v>
       </c>
       <c r="C37" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D37">
         <f t="shared" ca="1" si="6"/>
@@ -41978,7 +42116,7 @@
         <v>127</v>
       </c>
       <c r="C38" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D38">
         <f t="shared" ca="1" si="6"/>
@@ -42098,7 +42236,7 @@
         <v>128</v>
       </c>
       <c r="C39" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D39">
         <f t="shared" ca="1" si="6"/>
@@ -42218,7 +42356,7 @@
         <v>129</v>
       </c>
       <c r="C40" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D40">
         <f t="shared" ca="1" si="6"/>
@@ -42338,7 +42476,7 @@
         <v>130</v>
       </c>
       <c r="C41" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D41">
         <f t="shared" ref="D41:R46" ca="1" si="10">SUMIFS( INDIRECT(CONCATENATE($C41,"!", $A41, ":", $A41)),  INDIRECT(CONCATENATE($C41, "!$4:$4")), D$1)</f>
@@ -42458,7 +42596,7 @@
         <v>131</v>
       </c>
       <c r="C42" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D42">
         <f t="shared" ca="1" si="10"/>
@@ -42578,7 +42716,7 @@
         <v>132</v>
       </c>
       <c r="C43" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D43">
         <f t="shared" ca="1" si="10"/>
@@ -42698,7 +42836,7 @@
         <v>133</v>
       </c>
       <c r="C44" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D44">
         <f t="shared" ca="1" si="10"/>
@@ -42818,7 +42956,7 @@
         <v>134</v>
       </c>
       <c r="C45" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D45">
         <f t="shared" ca="1" si="10"/>
@@ -42938,7 +43076,7 @@
         <v>135</v>
       </c>
       <c r="C46" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D46">
         <f t="shared" ca="1" si="10"/>
@@ -45865,10 +46003,16 @@
         <v>167</v>
       </c>
       <c r="J1" s="76"/>
+      <c r="L1" t="s">
+        <v>323</v>
+      </c>
+      <c r="M1" t="s">
+        <v>323</v>
+      </c>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="76" t="s">
-        <v>311</v>
+      <c r="A2" s="81" t="s">
+        <v>321</v>
       </c>
       <c r="B2" s="76"/>
       <c r="C2" s="76"/>
@@ -48188,7 +48332,7 @@
     </row>
     <row r="91" spans="1:7">
       <c r="A91" s="17" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="C91" s="19"/>
       <c r="D91" s="19"/>
@@ -50484,7 +50628,7 @@
     </row>
     <row r="180" spans="1:7">
       <c r="A180" s="17" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="C180" s="19"/>
       <c r="D180" s="19"/>
@@ -52789,27 +52933,27 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="2" spans="1:15" ht="24">
-      <c r="A2" s="89"/>
-      <c r="B2" s="90" t="s">
+      <c r="A2" s="79"/>
+      <c r="B2" s="80" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="89"/>
-      <c r="D2" s="89"/>
-      <c r="E2" s="89"/>
-      <c r="F2" s="89"/>
-      <c r="G2" s="89"/>
-      <c r="H2" s="89"/>
-      <c r="I2" s="89"/>
-      <c r="J2" s="89"/>
-      <c r="K2" s="89"/>
-      <c r="L2" s="89"/>
-      <c r="M2" s="89"/>
-      <c r="N2" s="89"/>
-      <c r="O2" s="89"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
+      <c r="I2" s="79"/>
+      <c r="J2" s="79"/>
+      <c r="K2" s="79"/>
+      <c r="L2" s="79"/>
+      <c r="M2" s="79"/>
+      <c r="N2" s="79"/>
+      <c r="O2" s="79"/>
     </row>
     <row r="4" spans="1:15">
       <c r="E4" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -52817,18 +52961,18 @@
         <v>165</v>
       </c>
       <c r="F6" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="G6" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
     </row>
     <row r="7" spans="1:15">
       <c r="F7" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="G7" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -52982,7 +53126,7 @@
         <v>0.10299999999999999</v>
       </c>
       <c r="G21" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
     </row>
     <row r="22" spans="5:7">
@@ -53120,23 +53264,23 @@
       </c>
     </row>
     <row r="36" spans="1:15" ht="24">
-      <c r="A36" s="89"/>
-      <c r="B36" s="90" t="s">
+      <c r="A36" s="79"/>
+      <c r="B36" s="80" t="s">
         <v>47</v>
       </c>
-      <c r="C36" s="89"/>
-      <c r="D36" s="89"/>
-      <c r="E36" s="89"/>
-      <c r="F36" s="89"/>
-      <c r="G36" s="89"/>
-      <c r="H36" s="89"/>
-      <c r="I36" s="89"/>
-      <c r="J36" s="89"/>
-      <c r="K36" s="89"/>
-      <c r="L36" s="89"/>
-      <c r="M36" s="89"/>
-      <c r="N36" s="89"/>
-      <c r="O36" s="89"/>
+      <c r="C36" s="79"/>
+      <c r="D36" s="79"/>
+      <c r="E36" s="79"/>
+      <c r="F36" s="79"/>
+      <c r="G36" s="79"/>
+      <c r="H36" s="79"/>
+      <c r="I36" s="79"/>
+      <c r="J36" s="79"/>
+      <c r="K36" s="79"/>
+      <c r="L36" s="79"/>
+      <c r="M36" s="79"/>
+      <c r="N36" s="79"/>
+      <c r="O36" s="79"/>
     </row>
     <row r="43" spans="1:15">
       <c r="B43">

</xml_diff>